<commit_message>
Deploy bot Yamaha no Render
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -1,67 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\yamaha-bot\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DE3495-675F-44FA-A914-B3D31CCFB10B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>TELEFONE</t>
-  </si>
-  <si>
-    <t>NOME</t>
-  </si>
-  <si>
-    <t>MODELO</t>
-  </si>
-  <si>
-    <t>STATUS DE ENVIO</t>
-  </si>
-  <si>
-    <t>DATA DE ENVIO</t>
-  </si>
-  <si>
-    <t>JOAO VICTOR CORREIA DA SILVA</t>
-  </si>
-  <si>
-    <t>FZ15</t>
-  </si>
-  <si>
-    <t>Periodo</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -79,23 +46,81 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -383,89 +408,77 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="45.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>NOME</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TELEFONE</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>MODELO</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Periodo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>STATUS DE ENVIO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>DATA DE ENVIO</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1">
-        <v>5594992370446</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="1"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>JOAO VICTOR CORREIA DA SILVA</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5594992370446</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FZ15</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>06/04/2026 15:15</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Integração IA Fase 1
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\yamaha-bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19125917-4A5D-4170-AF33-634DA4E5BDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B1E29D-3DD9-4AAA-895A-B64E5447CA1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>NOME</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>NIVEL_INTERESSE</t>
+  </si>
+  <si>
+    <t>CHASSI</t>
   </si>
 </sst>
 </file>
@@ -154,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -164,6 +167,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -468,24 +474,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P375"/>
+  <dimension ref="A1:Q375"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="18.5546875" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="12.77734375" customWidth="1"/>
-    <col min="6" max="6" width="17.88671875" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" customWidth="1"/>
-    <col min="8" max="8" width="12.88671875" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" customWidth="1"/>
-    <col min="10" max="10" width="13.33203125" customWidth="1"/>
-    <col min="11" max="11" width="15.44140625" customWidth="1"/>
-    <col min="13" max="13" width="12.5546875" customWidth="1"/>
+    <col min="3" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="12.77734375" customWidth="1"/>
+    <col min="7" max="7" width="17.88671875" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" customWidth="1"/>
+    <col min="9" max="9" width="12.88671875" customWidth="1"/>
+    <col min="10" max="10" width="12.21875" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" customWidth="1"/>
+    <col min="14" max="14" width="12.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="41.4">
+    <row r="1" spans="1:17" ht="41.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -495,47 +501,50 @@
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:17">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -552,8 +561,9 @@
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
-    </row>
-    <row r="3" spans="1:16">
+      <c r="Q2" s="3"/>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -570,8 +580,9 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
-    </row>
-    <row r="4" spans="1:16">
+      <c r="Q3" s="3"/>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -588,8 +599,9 @@
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
-    </row>
-    <row r="5" spans="1:16">
+      <c r="Q4" s="3"/>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -606,8 +618,9 @@
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
-    </row>
-    <row r="6" spans="1:16">
+      <c r="Q5" s="3"/>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -624,8 +637,9 @@
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="Q6" s="3"/>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -642,8 +656,9 @@
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
-    </row>
-    <row r="8" spans="1:16">
+      <c r="Q7" s="3"/>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -660,8 +675,9 @@
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
-    </row>
-    <row r="9" spans="1:16">
+      <c r="Q8" s="3"/>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -678,8 +694,9 @@
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
-    </row>
-    <row r="10" spans="1:16">
+      <c r="Q9" s="3"/>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -696,8 +713,9 @@
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
-    </row>
-    <row r="11" spans="1:16">
+      <c r="Q10" s="3"/>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -714,8 +732,9 @@
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
-    </row>
-    <row r="12" spans="1:16">
+      <c r="Q11" s="3"/>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -732,8 +751,9 @@
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
-    </row>
-    <row r="13" spans="1:16">
+      <c r="Q12" s="3"/>
+    </row>
+    <row r="13" spans="1:17">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -750,8 +770,9 @@
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
-    </row>
-    <row r="14" spans="1:16">
+      <c r="Q13" s="3"/>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -768,8 +789,9 @@
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
-    </row>
-    <row r="15" spans="1:16">
+      <c r="Q14" s="3"/>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -786,8 +808,9 @@
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
-    </row>
-    <row r="16" spans="1:16">
+      <c r="Q15" s="3"/>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -804,8 +827,9 @@
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
-    </row>
-    <row r="17" spans="1:16">
+      <c r="Q16" s="3"/>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -822,8 +846,9 @@
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
-    </row>
-    <row r="18" spans="1:16">
+      <c r="Q17" s="3"/>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -840,8 +865,9 @@
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
-    </row>
-    <row r="19" spans="1:16">
+      <c r="Q18" s="3"/>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -858,8 +884,9 @@
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
       <c r="P19" s="3"/>
-    </row>
-    <row r="20" spans="1:16">
+      <c r="Q19" s="3"/>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -876,8 +903,9 @@
       <c r="N20" s="3"/>
       <c r="O20" s="3"/>
       <c r="P20" s="3"/>
-    </row>
-    <row r="21" spans="1:16">
+      <c r="Q20" s="3"/>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -894,8 +922,9 @@
       <c r="N21" s="3"/>
       <c r="O21" s="3"/>
       <c r="P21" s="3"/>
-    </row>
-    <row r="22" spans="1:16">
+      <c r="Q21" s="3"/>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -912,8 +941,9 @@
       <c r="N22" s="3"/>
       <c r="O22" s="3"/>
       <c r="P22" s="3"/>
-    </row>
-    <row r="23" spans="1:16">
+      <c r="Q22" s="3"/>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -930,8 +960,9 @@
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
-    </row>
-    <row r="24" spans="1:16">
+      <c r="Q23" s="3"/>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -948,8 +979,9 @@
       <c r="N24" s="3"/>
       <c r="O24" s="3"/>
       <c r="P24" s="3"/>
-    </row>
-    <row r="25" spans="1:16">
+      <c r="Q24" s="3"/>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -966,8 +998,9 @@
       <c r="N25" s="3"/>
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
-    </row>
-    <row r="26" spans="1:16">
+      <c r="Q25" s="3"/>
+    </row>
+    <row r="26" spans="1:17">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -984,8 +1017,9 @@
       <c r="N26" s="3"/>
       <c r="O26" s="3"/>
       <c r="P26" s="3"/>
-    </row>
-    <row r="27" spans="1:16">
+      <c r="Q26" s="3"/>
+    </row>
+    <row r="27" spans="1:17">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1002,8 +1036,9 @@
       <c r="N27" s="3"/>
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
-    </row>
-    <row r="28" spans="1:16">
+      <c r="Q27" s="3"/>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1020,8 +1055,9 @@
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
-    </row>
-    <row r="29" spans="1:16">
+      <c r="Q28" s="3"/>
+    </row>
+    <row r="29" spans="1:17">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1038,8 +1074,9 @@
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
-    </row>
-    <row r="30" spans="1:16">
+      <c r="Q29" s="3"/>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -1056,8 +1093,9 @@
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
-    </row>
-    <row r="31" spans="1:16">
+      <c r="Q30" s="3"/>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -1074,8 +1112,9 @@
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
-    </row>
-    <row r="32" spans="1:16">
+      <c r="Q31" s="3"/>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -1092,8 +1131,9 @@
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
-    </row>
-    <row r="33" spans="1:16">
+      <c r="Q32" s="3"/>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -1110,8 +1150,9 @@
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
-    </row>
-    <row r="34" spans="1:16">
+      <c r="Q33" s="3"/>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1128,8 +1169,9 @@
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
-    </row>
-    <row r="35" spans="1:16">
+      <c r="Q34" s="3"/>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -1146,8 +1188,9 @@
       <c r="N35" s="3"/>
       <c r="O35" s="3"/>
       <c r="P35" s="3"/>
-    </row>
-    <row r="36" spans="1:16">
+      <c r="Q35" s="3"/>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1164,8 +1207,9 @@
       <c r="N36" s="3"/>
       <c r="O36" s="3"/>
       <c r="P36" s="3"/>
-    </row>
-    <row r="37" spans="1:16">
+      <c r="Q36" s="3"/>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -1182,8 +1226,9 @@
       <c r="N37" s="3"/>
       <c r="O37" s="3"/>
       <c r="P37" s="3"/>
-    </row>
-    <row r="38" spans="1:16">
+      <c r="Q37" s="3"/>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1200,8 +1245,9 @@
       <c r="N38" s="3"/>
       <c r="O38" s="3"/>
       <c r="P38" s="3"/>
-    </row>
-    <row r="39" spans="1:16">
+      <c r="Q38" s="3"/>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -1218,8 +1264,9 @@
       <c r="N39" s="3"/>
       <c r="O39" s="3"/>
       <c r="P39" s="3"/>
-    </row>
-    <row r="40" spans="1:16">
+      <c r="Q39" s="3"/>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -1236,8 +1283,9 @@
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
-    </row>
-    <row r="41" spans="1:16">
+      <c r="Q40" s="3"/>
+    </row>
+    <row r="41" spans="1:17">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -1254,8 +1302,9 @@
       <c r="N41" s="3"/>
       <c r="O41" s="3"/>
       <c r="P41" s="3"/>
-    </row>
-    <row r="42" spans="1:16">
+      <c r="Q41" s="3"/>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -1272,8 +1321,9 @@
       <c r="N42" s="3"/>
       <c r="O42" s="3"/>
       <c r="P42" s="3"/>
-    </row>
-    <row r="43" spans="1:16">
+      <c r="Q42" s="3"/>
+    </row>
+    <row r="43" spans="1:17">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -1290,8 +1340,9 @@
       <c r="N43" s="3"/>
       <c r="O43" s="3"/>
       <c r="P43" s="3"/>
-    </row>
-    <row r="44" spans="1:16">
+      <c r="Q43" s="3"/>
+    </row>
+    <row r="44" spans="1:17">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1308,8 +1359,9 @@
       <c r="N44" s="3"/>
       <c r="O44" s="3"/>
       <c r="P44" s="3"/>
-    </row>
-    <row r="45" spans="1:16">
+      <c r="Q44" s="3"/>
+    </row>
+    <row r="45" spans="1:17">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -1326,8 +1378,9 @@
       <c r="N45" s="3"/>
       <c r="O45" s="3"/>
       <c r="P45" s="3"/>
-    </row>
-    <row r="46" spans="1:16">
+      <c r="Q45" s="3"/>
+    </row>
+    <row r="46" spans="1:17">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -1344,8 +1397,9 @@
       <c r="N46" s="3"/>
       <c r="O46" s="3"/>
       <c r="P46" s="3"/>
-    </row>
-    <row r="47" spans="1:16">
+      <c r="Q46" s="3"/>
+    </row>
+    <row r="47" spans="1:17">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
@@ -1362,8 +1416,9 @@
       <c r="N47" s="3"/>
       <c r="O47" s="3"/>
       <c r="P47" s="3"/>
-    </row>
-    <row r="48" spans="1:16">
+      <c r="Q47" s="3"/>
+    </row>
+    <row r="48" spans="1:17">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -1380,8 +1435,9 @@
       <c r="N48" s="3"/>
       <c r="O48" s="3"/>
       <c r="P48" s="3"/>
-    </row>
-    <row r="49" spans="1:16">
+      <c r="Q48" s="3"/>
+    </row>
+    <row r="49" spans="1:17">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -1398,8 +1454,9 @@
       <c r="N49" s="3"/>
       <c r="O49" s="3"/>
       <c r="P49" s="3"/>
-    </row>
-    <row r="50" spans="1:16">
+      <c r="Q49" s="3"/>
+    </row>
+    <row r="50" spans="1:17">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -1416,8 +1473,9 @@
       <c r="N50" s="3"/>
       <c r="O50" s="3"/>
       <c r="P50" s="3"/>
-    </row>
-    <row r="51" spans="1:16">
+      <c r="Q50" s="3"/>
+    </row>
+    <row r="51" spans="1:17">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
@@ -1434,8 +1492,9 @@
       <c r="N51" s="3"/>
       <c r="O51" s="3"/>
       <c r="P51" s="3"/>
-    </row>
-    <row r="52" spans="1:16">
+      <c r="Q51" s="3"/>
+    </row>
+    <row r="52" spans="1:17">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -1452,8 +1511,9 @@
       <c r="N52" s="3"/>
       <c r="O52" s="3"/>
       <c r="P52" s="3"/>
-    </row>
-    <row r="53" spans="1:16">
+      <c r="Q52" s="3"/>
+    </row>
+    <row r="53" spans="1:17">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
@@ -1470,8 +1530,9 @@
       <c r="N53" s="3"/>
       <c r="O53" s="3"/>
       <c r="P53" s="3"/>
-    </row>
-    <row r="54" spans="1:16">
+      <c r="Q53" s="3"/>
+    </row>
+    <row r="54" spans="1:17">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -1488,8 +1549,9 @@
       <c r="N54" s="3"/>
       <c r="O54" s="3"/>
       <c r="P54" s="3"/>
-    </row>
-    <row r="55" spans="1:16">
+      <c r="Q54" s="3"/>
+    </row>
+    <row r="55" spans="1:17">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -1506,8 +1568,9 @@
       <c r="N55" s="3"/>
       <c r="O55" s="3"/>
       <c r="P55" s="3"/>
-    </row>
-    <row r="56" spans="1:16">
+      <c r="Q55" s="3"/>
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -1524,8 +1587,9 @@
       <c r="N56" s="3"/>
       <c r="O56" s="3"/>
       <c r="P56" s="3"/>
-    </row>
-    <row r="57" spans="1:16">
+      <c r="Q56" s="3"/>
+    </row>
+    <row r="57" spans="1:17">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -1542,8 +1606,9 @@
       <c r="N57" s="3"/>
       <c r="O57" s="3"/>
       <c r="P57" s="3"/>
-    </row>
-    <row r="58" spans="1:16">
+      <c r="Q57" s="3"/>
+    </row>
+    <row r="58" spans="1:17">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -1560,8 +1625,9 @@
       <c r="N58" s="3"/>
       <c r="O58" s="3"/>
       <c r="P58" s="3"/>
-    </row>
-    <row r="59" spans="1:16">
+      <c r="Q58" s="3"/>
+    </row>
+    <row r="59" spans="1:17">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -1578,8 +1644,9 @@
       <c r="N59" s="3"/>
       <c r="O59" s="3"/>
       <c r="P59" s="3"/>
-    </row>
-    <row r="60" spans="1:16">
+      <c r="Q59" s="3"/>
+    </row>
+    <row r="60" spans="1:17">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -1596,8 +1663,9 @@
       <c r="N60" s="3"/>
       <c r="O60" s="3"/>
       <c r="P60" s="3"/>
-    </row>
-    <row r="61" spans="1:16">
+      <c r="Q60" s="3"/>
+    </row>
+    <row r="61" spans="1:17">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -1614,8 +1682,9 @@
       <c r="N61" s="3"/>
       <c r="O61" s="3"/>
       <c r="P61" s="3"/>
-    </row>
-    <row r="62" spans="1:16">
+      <c r="Q61" s="3"/>
+    </row>
+    <row r="62" spans="1:17">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -1632,8 +1701,9 @@
       <c r="N62" s="3"/>
       <c r="O62" s="3"/>
       <c r="P62" s="3"/>
-    </row>
-    <row r="63" spans="1:16">
+      <c r="Q62" s="3"/>
+    </row>
+    <row r="63" spans="1:17">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -1650,8 +1720,9 @@
       <c r="N63" s="3"/>
       <c r="O63" s="3"/>
       <c r="P63" s="3"/>
-    </row>
-    <row r="64" spans="1:16">
+      <c r="Q63" s="3"/>
+    </row>
+    <row r="64" spans="1:17">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -1668,8 +1739,9 @@
       <c r="N64" s="3"/>
       <c r="O64" s="3"/>
       <c r="P64" s="3"/>
-    </row>
-    <row r="65" spans="1:16">
+      <c r="Q64" s="3"/>
+    </row>
+    <row r="65" spans="1:17">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
@@ -1686,8 +1758,9 @@
       <c r="N65" s="3"/>
       <c r="O65" s="3"/>
       <c r="P65" s="3"/>
-    </row>
-    <row r="66" spans="1:16">
+      <c r="Q65" s="3"/>
+    </row>
+    <row r="66" spans="1:17">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -1704,8 +1777,9 @@
       <c r="N66" s="3"/>
       <c r="O66" s="3"/>
       <c r="P66" s="3"/>
-    </row>
-    <row r="67" spans="1:16">
+      <c r="Q66" s="3"/>
+    </row>
+    <row r="67" spans="1:17">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -1722,8 +1796,9 @@
       <c r="N67" s="3"/>
       <c r="O67" s="3"/>
       <c r="P67" s="3"/>
-    </row>
-    <row r="68" spans="1:16">
+      <c r="Q67" s="3"/>
+    </row>
+    <row r="68" spans="1:17">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -1740,8 +1815,9 @@
       <c r="N68" s="3"/>
       <c r="O68" s="3"/>
       <c r="P68" s="3"/>
-    </row>
-    <row r="69" spans="1:16">
+      <c r="Q68" s="3"/>
+    </row>
+    <row r="69" spans="1:17">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
@@ -1758,8 +1834,9 @@
       <c r="N69" s="3"/>
       <c r="O69" s="3"/>
       <c r="P69" s="3"/>
-    </row>
-    <row r="70" spans="1:16">
+      <c r="Q69" s="3"/>
+    </row>
+    <row r="70" spans="1:17">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -1776,8 +1853,9 @@
       <c r="N70" s="3"/>
       <c r="O70" s="3"/>
       <c r="P70" s="3"/>
-    </row>
-    <row r="71" spans="1:16">
+      <c r="Q70" s="3"/>
+    </row>
+    <row r="71" spans="1:17">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
@@ -1794,8 +1872,9 @@
       <c r="N71" s="3"/>
       <c r="O71" s="3"/>
       <c r="P71" s="3"/>
-    </row>
-    <row r="72" spans="1:16">
+      <c r="Q71" s="3"/>
+    </row>
+    <row r="72" spans="1:17">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -1812,8 +1891,9 @@
       <c r="N72" s="3"/>
       <c r="O72" s="3"/>
       <c r="P72" s="3"/>
-    </row>
-    <row r="73" spans="1:16">
+      <c r="Q72" s="3"/>
+    </row>
+    <row r="73" spans="1:17">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -1830,8 +1910,9 @@
       <c r="N73" s="3"/>
       <c r="O73" s="3"/>
       <c r="P73" s="3"/>
-    </row>
-    <row r="74" spans="1:16">
+      <c r="Q73" s="3"/>
+    </row>
+    <row r="74" spans="1:17">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -1848,8 +1929,9 @@
       <c r="N74" s="3"/>
       <c r="O74" s="3"/>
       <c r="P74" s="3"/>
-    </row>
-    <row r="75" spans="1:16">
+      <c r="Q74" s="3"/>
+    </row>
+    <row r="75" spans="1:17">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -1866,8 +1948,9 @@
       <c r="N75" s="3"/>
       <c r="O75" s="3"/>
       <c r="P75" s="3"/>
-    </row>
-    <row r="76" spans="1:16">
+      <c r="Q75" s="3"/>
+    </row>
+    <row r="76" spans="1:17">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -1884,8 +1967,9 @@
       <c r="N76" s="3"/>
       <c r="O76" s="3"/>
       <c r="P76" s="3"/>
-    </row>
-    <row r="77" spans="1:16">
+      <c r="Q76" s="3"/>
+    </row>
+    <row r="77" spans="1:17">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -1902,8 +1986,9 @@
       <c r="N77" s="3"/>
       <c r="O77" s="3"/>
       <c r="P77" s="3"/>
-    </row>
-    <row r="78" spans="1:16">
+      <c r="Q77" s="3"/>
+    </row>
+    <row r="78" spans="1:17">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -1920,8 +2005,9 @@
       <c r="N78" s="3"/>
       <c r="O78" s="3"/>
       <c r="P78" s="3"/>
-    </row>
-    <row r="79" spans="1:16">
+      <c r="Q78" s="3"/>
+    </row>
+    <row r="79" spans="1:17">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
@@ -1938,8 +2024,9 @@
       <c r="N79" s="3"/>
       <c r="O79" s="3"/>
       <c r="P79" s="3"/>
-    </row>
-    <row r="80" spans="1:16">
+      <c r="Q79" s="3"/>
+    </row>
+    <row r="80" spans="1:17">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -1956,8 +2043,9 @@
       <c r="N80" s="3"/>
       <c r="O80" s="3"/>
       <c r="P80" s="3"/>
-    </row>
-    <row r="81" spans="1:16">
+      <c r="Q80" s="3"/>
+    </row>
+    <row r="81" spans="1:17">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
@@ -1974,8 +2062,9 @@
       <c r="N81" s="3"/>
       <c r="O81" s="3"/>
       <c r="P81" s="3"/>
-    </row>
-    <row r="82" spans="1:16">
+      <c r="Q81" s="3"/>
+    </row>
+    <row r="82" spans="1:17">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -1992,8 +2081,9 @@
       <c r="N82" s="3"/>
       <c r="O82" s="3"/>
       <c r="P82" s="3"/>
-    </row>
-    <row r="83" spans="1:16">
+      <c r="Q82" s="3"/>
+    </row>
+    <row r="83" spans="1:17">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -2010,8 +2100,9 @@
       <c r="N83" s="3"/>
       <c r="O83" s="3"/>
       <c r="P83" s="3"/>
-    </row>
-    <row r="84" spans="1:16">
+      <c r="Q83" s="3"/>
+    </row>
+    <row r="84" spans="1:17">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -2028,8 +2119,9 @@
       <c r="N84" s="3"/>
       <c r="O84" s="3"/>
       <c r="P84" s="3"/>
-    </row>
-    <row r="85" spans="1:16">
+      <c r="Q84" s="3"/>
+    </row>
+    <row r="85" spans="1:17">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
@@ -2046,8 +2138,9 @@
       <c r="N85" s="3"/>
       <c r="O85" s="3"/>
       <c r="P85" s="3"/>
-    </row>
-    <row r="86" spans="1:16">
+      <c r="Q85" s="3"/>
+    </row>
+    <row r="86" spans="1:17">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -2064,8 +2157,9 @@
       <c r="N86" s="3"/>
       <c r="O86" s="3"/>
       <c r="P86" s="3"/>
-    </row>
-    <row r="87" spans="1:16">
+      <c r="Q86" s="3"/>
+    </row>
+    <row r="87" spans="1:17">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -2082,8 +2176,9 @@
       <c r="N87" s="3"/>
       <c r="O87" s="3"/>
       <c r="P87" s="3"/>
-    </row>
-    <row r="88" spans="1:16">
+      <c r="Q87" s="3"/>
+    </row>
+    <row r="88" spans="1:17">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -2100,8 +2195,9 @@
       <c r="N88" s="3"/>
       <c r="O88" s="3"/>
       <c r="P88" s="3"/>
-    </row>
-    <row r="89" spans="1:16">
+      <c r="Q88" s="3"/>
+    </row>
+    <row r="89" spans="1:17">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
@@ -2118,8 +2214,9 @@
       <c r="N89" s="3"/>
       <c r="O89" s="3"/>
       <c r="P89" s="3"/>
-    </row>
-    <row r="90" spans="1:16">
+      <c r="Q89" s="3"/>
+    </row>
+    <row r="90" spans="1:17">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -2136,8 +2233,9 @@
       <c r="N90" s="3"/>
       <c r="O90" s="3"/>
       <c r="P90" s="3"/>
-    </row>
-    <row r="91" spans="1:16">
+      <c r="Q90" s="3"/>
+    </row>
+    <row r="91" spans="1:17">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
@@ -2154,8 +2252,9 @@
       <c r="N91" s="3"/>
       <c r="O91" s="3"/>
       <c r="P91" s="3"/>
-    </row>
-    <row r="92" spans="1:16">
+      <c r="Q91" s="3"/>
+    </row>
+    <row r="92" spans="1:17">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -2172,8 +2271,9 @@
       <c r="N92" s="3"/>
       <c r="O92" s="3"/>
       <c r="P92" s="3"/>
-    </row>
-    <row r="93" spans="1:16">
+      <c r="Q92" s="3"/>
+    </row>
+    <row r="93" spans="1:17">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
@@ -2190,8 +2290,9 @@
       <c r="N93" s="3"/>
       <c r="O93" s="3"/>
       <c r="P93" s="3"/>
-    </row>
-    <row r="94" spans="1:16">
+      <c r="Q93" s="3"/>
+    </row>
+    <row r="94" spans="1:17">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -2208,8 +2309,9 @@
       <c r="N94" s="3"/>
       <c r="O94" s="3"/>
       <c r="P94" s="3"/>
-    </row>
-    <row r="95" spans="1:16">
+      <c r="Q94" s="3"/>
+    </row>
+    <row r="95" spans="1:17">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
@@ -2226,8 +2328,9 @@
       <c r="N95" s="3"/>
       <c r="O95" s="3"/>
       <c r="P95" s="3"/>
-    </row>
-    <row r="96" spans="1:16">
+      <c r="Q95" s="3"/>
+    </row>
+    <row r="96" spans="1:17">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -2244,8 +2347,9 @@
       <c r="N96" s="3"/>
       <c r="O96" s="3"/>
       <c r="P96" s="3"/>
-    </row>
-    <row r="97" spans="1:16">
+      <c r="Q96" s="3"/>
+    </row>
+    <row r="97" spans="1:17">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
@@ -2262,8 +2366,9 @@
       <c r="N97" s="3"/>
       <c r="O97" s="3"/>
       <c r="P97" s="3"/>
-    </row>
-    <row r="98" spans="1:16">
+      <c r="Q97" s="3"/>
+    </row>
+    <row r="98" spans="1:17">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -2280,8 +2385,9 @@
       <c r="N98" s="3"/>
       <c r="O98" s="3"/>
       <c r="P98" s="3"/>
-    </row>
-    <row r="99" spans="1:16">
+      <c r="Q98" s="3"/>
+    </row>
+    <row r="99" spans="1:17">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
@@ -2298,8 +2404,9 @@
       <c r="N99" s="3"/>
       <c r="O99" s="3"/>
       <c r="P99" s="3"/>
-    </row>
-    <row r="100" spans="1:16">
+      <c r="Q99" s="3"/>
+    </row>
+    <row r="100" spans="1:17">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -2316,8 +2423,9 @@
       <c r="N100" s="3"/>
       <c r="O100" s="3"/>
       <c r="P100" s="3"/>
-    </row>
-    <row r="101" spans="1:16">
+      <c r="Q100" s="3"/>
+    </row>
+    <row r="101" spans="1:17">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -2334,8 +2442,9 @@
       <c r="N101" s="3"/>
       <c r="O101" s="3"/>
       <c r="P101" s="3"/>
-    </row>
-    <row r="102" spans="1:16">
+      <c r="Q101" s="3"/>
+    </row>
+    <row r="102" spans="1:17">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
@@ -2352,8 +2461,9 @@
       <c r="N102" s="3"/>
       <c r="O102" s="3"/>
       <c r="P102" s="3"/>
-    </row>
-    <row r="103" spans="1:16">
+      <c r="Q102" s="3"/>
+    </row>
+    <row r="103" spans="1:17">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
@@ -2370,8 +2480,9 @@
       <c r="N103" s="3"/>
       <c r="O103" s="3"/>
       <c r="P103" s="3"/>
-    </row>
-    <row r="104" spans="1:16">
+      <c r="Q103" s="3"/>
+    </row>
+    <row r="104" spans="1:17">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
@@ -2388,8 +2499,9 @@
       <c r="N104" s="3"/>
       <c r="O104" s="3"/>
       <c r="P104" s="3"/>
-    </row>
-    <row r="105" spans="1:16">
+      <c r="Q104" s="3"/>
+    </row>
+    <row r="105" spans="1:17">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
@@ -2406,8 +2518,9 @@
       <c r="N105" s="3"/>
       <c r="O105" s="3"/>
       <c r="P105" s="3"/>
-    </row>
-    <row r="106" spans="1:16">
+      <c r="Q105" s="3"/>
+    </row>
+    <row r="106" spans="1:17">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
@@ -2424,8 +2537,9 @@
       <c r="N106" s="3"/>
       <c r="O106" s="3"/>
       <c r="P106" s="3"/>
-    </row>
-    <row r="107" spans="1:16">
+      <c r="Q106" s="3"/>
+    </row>
+    <row r="107" spans="1:17">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
@@ -2442,8 +2556,9 @@
       <c r="N107" s="3"/>
       <c r="O107" s="3"/>
       <c r="P107" s="3"/>
-    </row>
-    <row r="108" spans="1:16">
+      <c r="Q107" s="3"/>
+    </row>
+    <row r="108" spans="1:17">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
@@ -2460,8 +2575,9 @@
       <c r="N108" s="3"/>
       <c r="O108" s="3"/>
       <c r="P108" s="3"/>
-    </row>
-    <row r="109" spans="1:16">
+      <c r="Q108" s="3"/>
+    </row>
+    <row r="109" spans="1:17">
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
@@ -2478,8 +2594,9 @@
       <c r="N109" s="3"/>
       <c r="O109" s="3"/>
       <c r="P109" s="3"/>
-    </row>
-    <row r="110" spans="1:16">
+      <c r="Q109" s="3"/>
+    </row>
+    <row r="110" spans="1:17">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
@@ -2496,8 +2613,9 @@
       <c r="N110" s="3"/>
       <c r="O110" s="3"/>
       <c r="P110" s="3"/>
-    </row>
-    <row r="111" spans="1:16">
+      <c r="Q110" s="3"/>
+    </row>
+    <row r="111" spans="1:17">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
@@ -2514,8 +2632,9 @@
       <c r="N111" s="3"/>
       <c r="O111" s="3"/>
       <c r="P111" s="3"/>
-    </row>
-    <row r="112" spans="1:16">
+      <c r="Q111" s="3"/>
+    </row>
+    <row r="112" spans="1:17">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
@@ -2532,8 +2651,9 @@
       <c r="N112" s="3"/>
       <c r="O112" s="3"/>
       <c r="P112" s="3"/>
-    </row>
-    <row r="113" spans="1:16">
+      <c r="Q112" s="3"/>
+    </row>
+    <row r="113" spans="1:17">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
@@ -2550,8 +2670,9 @@
       <c r="N113" s="3"/>
       <c r="O113" s="3"/>
       <c r="P113" s="3"/>
-    </row>
-    <row r="114" spans="1:16">
+      <c r="Q113" s="3"/>
+    </row>
+    <row r="114" spans="1:17">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
@@ -2568,8 +2689,9 @@
       <c r="N114" s="3"/>
       <c r="O114" s="3"/>
       <c r="P114" s="3"/>
-    </row>
-    <row r="115" spans="1:16">
+      <c r="Q114" s="3"/>
+    </row>
+    <row r="115" spans="1:17">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
@@ -2586,8 +2708,9 @@
       <c r="N115" s="3"/>
       <c r="O115" s="3"/>
       <c r="P115" s="3"/>
-    </row>
-    <row r="116" spans="1:16">
+      <c r="Q115" s="3"/>
+    </row>
+    <row r="116" spans="1:17">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
@@ -2604,8 +2727,9 @@
       <c r="N116" s="3"/>
       <c r="O116" s="3"/>
       <c r="P116" s="3"/>
-    </row>
-    <row r="117" spans="1:16">
+      <c r="Q116" s="3"/>
+    </row>
+    <row r="117" spans="1:17">
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
@@ -2622,8 +2746,9 @@
       <c r="N117" s="3"/>
       <c r="O117" s="3"/>
       <c r="P117" s="3"/>
-    </row>
-    <row r="118" spans="1:16">
+      <c r="Q117" s="3"/>
+    </row>
+    <row r="118" spans="1:17">
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
@@ -2640,8 +2765,9 @@
       <c r="N118" s="3"/>
       <c r="O118" s="3"/>
       <c r="P118" s="3"/>
-    </row>
-    <row r="119" spans="1:16">
+      <c r="Q118" s="3"/>
+    </row>
+    <row r="119" spans="1:17">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
@@ -2658,8 +2784,9 @@
       <c r="N119" s="3"/>
       <c r="O119" s="3"/>
       <c r="P119" s="3"/>
-    </row>
-    <row r="120" spans="1:16">
+      <c r="Q119" s="3"/>
+    </row>
+    <row r="120" spans="1:17">
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
@@ -2676,8 +2803,9 @@
       <c r="N120" s="3"/>
       <c r="O120" s="3"/>
       <c r="P120" s="3"/>
-    </row>
-    <row r="121" spans="1:16">
+      <c r="Q120" s="3"/>
+    </row>
+    <row r="121" spans="1:17">
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
@@ -2694,8 +2822,9 @@
       <c r="N121" s="3"/>
       <c r="O121" s="3"/>
       <c r="P121" s="3"/>
-    </row>
-    <row r="122" spans="1:16">
+      <c r="Q121" s="3"/>
+    </row>
+    <row r="122" spans="1:17">
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
@@ -2712,8 +2841,9 @@
       <c r="N122" s="3"/>
       <c r="O122" s="3"/>
       <c r="P122" s="3"/>
-    </row>
-    <row r="123" spans="1:16">
+      <c r="Q122" s="3"/>
+    </row>
+    <row r="123" spans="1:17">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
@@ -2730,8 +2860,9 @@
       <c r="N123" s="3"/>
       <c r="O123" s="3"/>
       <c r="P123" s="3"/>
-    </row>
-    <row r="124" spans="1:16">
+      <c r="Q123" s="3"/>
+    </row>
+    <row r="124" spans="1:17">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
@@ -2748,8 +2879,9 @@
       <c r="N124" s="3"/>
       <c r="O124" s="3"/>
       <c r="P124" s="3"/>
-    </row>
-    <row r="125" spans="1:16">
+      <c r="Q124" s="3"/>
+    </row>
+    <row r="125" spans="1:17">
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
@@ -2766,8 +2898,9 @@
       <c r="N125" s="3"/>
       <c r="O125" s="3"/>
       <c r="P125" s="3"/>
-    </row>
-    <row r="126" spans="1:16">
+      <c r="Q125" s="3"/>
+    </row>
+    <row r="126" spans="1:17">
       <c r="A126" s="3"/>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
@@ -2784,8 +2917,9 @@
       <c r="N126" s="3"/>
       <c r="O126" s="3"/>
       <c r="P126" s="3"/>
-    </row>
-    <row r="127" spans="1:16">
+      <c r="Q126" s="3"/>
+    </row>
+    <row r="127" spans="1:17">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
@@ -2802,8 +2936,9 @@
       <c r="N127" s="3"/>
       <c r="O127" s="3"/>
       <c r="P127" s="3"/>
-    </row>
-    <row r="128" spans="1:16">
+      <c r="Q127" s="3"/>
+    </row>
+    <row r="128" spans="1:17">
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
@@ -2820,8 +2955,9 @@
       <c r="N128" s="3"/>
       <c r="O128" s="3"/>
       <c r="P128" s="3"/>
-    </row>
-    <row r="129" spans="1:16">
+      <c r="Q128" s="3"/>
+    </row>
+    <row r="129" spans="1:17">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
@@ -2838,8 +2974,9 @@
       <c r="N129" s="3"/>
       <c r="O129" s="3"/>
       <c r="P129" s="3"/>
-    </row>
-    <row r="130" spans="1:16">
+      <c r="Q129" s="3"/>
+    </row>
+    <row r="130" spans="1:17">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
@@ -2856,8 +2993,9 @@
       <c r="N130" s="3"/>
       <c r="O130" s="3"/>
       <c r="P130" s="3"/>
-    </row>
-    <row r="131" spans="1:16">
+      <c r="Q130" s="3"/>
+    </row>
+    <row r="131" spans="1:17">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
@@ -2874,8 +3012,9 @@
       <c r="N131" s="3"/>
       <c r="O131" s="3"/>
       <c r="P131" s="3"/>
-    </row>
-    <row r="132" spans="1:16">
+      <c r="Q131" s="3"/>
+    </row>
+    <row r="132" spans="1:17">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
@@ -2892,8 +3031,9 @@
       <c r="N132" s="3"/>
       <c r="O132" s="3"/>
       <c r="P132" s="3"/>
-    </row>
-    <row r="133" spans="1:16">
+      <c r="Q132" s="3"/>
+    </row>
+    <row r="133" spans="1:17">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
@@ -2910,8 +3050,9 @@
       <c r="N133" s="3"/>
       <c r="O133" s="3"/>
       <c r="P133" s="3"/>
-    </row>
-    <row r="134" spans="1:16">
+      <c r="Q133" s="3"/>
+    </row>
+    <row r="134" spans="1:17">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
@@ -2928,8 +3069,9 @@
       <c r="N134" s="3"/>
       <c r="O134" s="3"/>
       <c r="P134" s="3"/>
-    </row>
-    <row r="135" spans="1:16">
+      <c r="Q134" s="3"/>
+    </row>
+    <row r="135" spans="1:17">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
@@ -2946,8 +3088,9 @@
       <c r="N135" s="3"/>
       <c r="O135" s="3"/>
       <c r="P135" s="3"/>
-    </row>
-    <row r="136" spans="1:16">
+      <c r="Q135" s="3"/>
+    </row>
+    <row r="136" spans="1:17">
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
@@ -2964,8 +3107,9 @@
       <c r="N136" s="3"/>
       <c r="O136" s="3"/>
       <c r="P136" s="3"/>
-    </row>
-    <row r="137" spans="1:16">
+      <c r="Q136" s="3"/>
+    </row>
+    <row r="137" spans="1:17">
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
@@ -2982,8 +3126,9 @@
       <c r="N137" s="3"/>
       <c r="O137" s="3"/>
       <c r="P137" s="3"/>
-    </row>
-    <row r="138" spans="1:16">
+      <c r="Q137" s="3"/>
+    </row>
+    <row r="138" spans="1:17">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
@@ -3000,8 +3145,9 @@
       <c r="N138" s="3"/>
       <c r="O138" s="3"/>
       <c r="P138" s="3"/>
-    </row>
-    <row r="139" spans="1:16">
+      <c r="Q138" s="3"/>
+    </row>
+    <row r="139" spans="1:17">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
@@ -3018,8 +3164,9 @@
       <c r="N139" s="3"/>
       <c r="O139" s="3"/>
       <c r="P139" s="3"/>
-    </row>
-    <row r="140" spans="1:16">
+      <c r="Q139" s="3"/>
+    </row>
+    <row r="140" spans="1:17">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
@@ -3036,8 +3183,9 @@
       <c r="N140" s="3"/>
       <c r="O140" s="3"/>
       <c r="P140" s="3"/>
-    </row>
-    <row r="141" spans="1:16">
+      <c r="Q140" s="3"/>
+    </row>
+    <row r="141" spans="1:17">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
@@ -3054,8 +3202,9 @@
       <c r="N141" s="3"/>
       <c r="O141" s="3"/>
       <c r="P141" s="3"/>
-    </row>
-    <row r="142" spans="1:16">
+      <c r="Q141" s="3"/>
+    </row>
+    <row r="142" spans="1:17">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
@@ -3072,8 +3221,9 @@
       <c r="N142" s="3"/>
       <c r="O142" s="3"/>
       <c r="P142" s="3"/>
-    </row>
-    <row r="143" spans="1:16">
+      <c r="Q142" s="3"/>
+    </row>
+    <row r="143" spans="1:17">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
@@ -3090,8 +3240,9 @@
       <c r="N143" s="3"/>
       <c r="O143" s="3"/>
       <c r="P143" s="3"/>
-    </row>
-    <row r="144" spans="1:16">
+      <c r="Q143" s="3"/>
+    </row>
+    <row r="144" spans="1:17">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
@@ -3108,8 +3259,9 @@
       <c r="N144" s="3"/>
       <c r="O144" s="3"/>
       <c r="P144" s="3"/>
-    </row>
-    <row r="145" spans="1:16">
+      <c r="Q144" s="3"/>
+    </row>
+    <row r="145" spans="1:17">
       <c r="A145" s="3"/>
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
@@ -3126,8 +3278,9 @@
       <c r="N145" s="3"/>
       <c r="O145" s="3"/>
       <c r="P145" s="3"/>
-    </row>
-    <row r="146" spans="1:16">
+      <c r="Q145" s="3"/>
+    </row>
+    <row r="146" spans="1:17">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
@@ -3144,8 +3297,9 @@
       <c r="N146" s="3"/>
       <c r="O146" s="3"/>
       <c r="P146" s="3"/>
-    </row>
-    <row r="147" spans="1:16">
+      <c r="Q146" s="3"/>
+    </row>
+    <row r="147" spans="1:17">
       <c r="A147" s="3"/>
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
@@ -3162,8 +3316,9 @@
       <c r="N147" s="3"/>
       <c r="O147" s="3"/>
       <c r="P147" s="3"/>
-    </row>
-    <row r="148" spans="1:16">
+      <c r="Q147" s="3"/>
+    </row>
+    <row r="148" spans="1:17">
       <c r="A148" s="3"/>
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
@@ -3180,8 +3335,9 @@
       <c r="N148" s="3"/>
       <c r="O148" s="3"/>
       <c r="P148" s="3"/>
-    </row>
-    <row r="149" spans="1:16">
+      <c r="Q148" s="3"/>
+    </row>
+    <row r="149" spans="1:17">
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
@@ -3198,8 +3354,9 @@
       <c r="N149" s="3"/>
       <c r="O149" s="3"/>
       <c r="P149" s="3"/>
-    </row>
-    <row r="150" spans="1:16">
+      <c r="Q149" s="3"/>
+    </row>
+    <row r="150" spans="1:17">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
@@ -3216,8 +3373,9 @@
       <c r="N150" s="3"/>
       <c r="O150" s="3"/>
       <c r="P150" s="3"/>
-    </row>
-    <row r="151" spans="1:16">
+      <c r="Q150" s="3"/>
+    </row>
+    <row r="151" spans="1:17">
       <c r="A151" s="3"/>
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
@@ -3234,8 +3392,9 @@
       <c r="N151" s="3"/>
       <c r="O151" s="3"/>
       <c r="P151" s="3"/>
-    </row>
-    <row r="152" spans="1:16">
+      <c r="Q151" s="3"/>
+    </row>
+    <row r="152" spans="1:17">
       <c r="A152" s="3"/>
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
@@ -3252,8 +3411,9 @@
       <c r="N152" s="3"/>
       <c r="O152" s="3"/>
       <c r="P152" s="3"/>
-    </row>
-    <row r="153" spans="1:16">
+      <c r="Q152" s="3"/>
+    </row>
+    <row r="153" spans="1:17">
       <c r="A153" s="3"/>
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
@@ -3270,8 +3430,9 @@
       <c r="N153" s="3"/>
       <c r="O153" s="3"/>
       <c r="P153" s="3"/>
-    </row>
-    <row r="154" spans="1:16">
+      <c r="Q153" s="3"/>
+    </row>
+    <row r="154" spans="1:17">
       <c r="A154" s="3"/>
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
@@ -3288,8 +3449,9 @@
       <c r="N154" s="3"/>
       <c r="O154" s="3"/>
       <c r="P154" s="3"/>
-    </row>
-    <row r="155" spans="1:16">
+      <c r="Q154" s="3"/>
+    </row>
+    <row r="155" spans="1:17">
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
@@ -3306,8 +3468,9 @@
       <c r="N155" s="3"/>
       <c r="O155" s="3"/>
       <c r="P155" s="3"/>
-    </row>
-    <row r="156" spans="1:16">
+      <c r="Q155" s="3"/>
+    </row>
+    <row r="156" spans="1:17">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
@@ -3324,8 +3487,9 @@
       <c r="N156" s="3"/>
       <c r="O156" s="3"/>
       <c r="P156" s="3"/>
-    </row>
-    <row r="157" spans="1:16">
+      <c r="Q156" s="3"/>
+    </row>
+    <row r="157" spans="1:17">
       <c r="A157" s="3"/>
       <c r="B157" s="3"/>
       <c r="C157" s="3"/>
@@ -3342,8 +3506,9 @@
       <c r="N157" s="3"/>
       <c r="O157" s="3"/>
       <c r="P157" s="3"/>
-    </row>
-    <row r="158" spans="1:16">
+      <c r="Q157" s="3"/>
+    </row>
+    <row r="158" spans="1:17">
       <c r="A158" s="3"/>
       <c r="B158" s="3"/>
       <c r="C158" s="3"/>
@@ -3360,8 +3525,9 @@
       <c r="N158" s="3"/>
       <c r="O158" s="3"/>
       <c r="P158" s="3"/>
-    </row>
-    <row r="159" spans="1:16">
+      <c r="Q158" s="3"/>
+    </row>
+    <row r="159" spans="1:17">
       <c r="A159" s="3"/>
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
@@ -3378,8 +3544,9 @@
       <c r="N159" s="3"/>
       <c r="O159" s="3"/>
       <c r="P159" s="3"/>
-    </row>
-    <row r="160" spans="1:16">
+      <c r="Q159" s="3"/>
+    </row>
+    <row r="160" spans="1:17">
       <c r="A160" s="3"/>
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
@@ -3396,8 +3563,9 @@
       <c r="N160" s="3"/>
       <c r="O160" s="3"/>
       <c r="P160" s="3"/>
-    </row>
-    <row r="161" spans="1:16">
+      <c r="Q160" s="3"/>
+    </row>
+    <row r="161" spans="1:17">
       <c r="A161" s="3"/>
       <c r="B161" s="3"/>
       <c r="C161" s="3"/>
@@ -3414,8 +3582,9 @@
       <c r="N161" s="3"/>
       <c r="O161" s="3"/>
       <c r="P161" s="3"/>
-    </row>
-    <row r="162" spans="1:16">
+      <c r="Q161" s="3"/>
+    </row>
+    <row r="162" spans="1:17">
       <c r="A162" s="3"/>
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
@@ -3432,8 +3601,9 @@
       <c r="N162" s="3"/>
       <c r="O162" s="3"/>
       <c r="P162" s="3"/>
-    </row>
-    <row r="163" spans="1:16">
+      <c r="Q162" s="3"/>
+    </row>
+    <row r="163" spans="1:17">
       <c r="A163" s="3"/>
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
@@ -3450,8 +3620,9 @@
       <c r="N163" s="3"/>
       <c r="O163" s="3"/>
       <c r="P163" s="3"/>
-    </row>
-    <row r="164" spans="1:16">
+      <c r="Q163" s="3"/>
+    </row>
+    <row r="164" spans="1:17">
       <c r="A164" s="3"/>
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
@@ -3468,8 +3639,9 @@
       <c r="N164" s="3"/>
       <c r="O164" s="3"/>
       <c r="P164" s="3"/>
-    </row>
-    <row r="165" spans="1:16">
+      <c r="Q164" s="3"/>
+    </row>
+    <row r="165" spans="1:17">
       <c r="A165" s="3"/>
       <c r="B165" s="3"/>
       <c r="C165" s="3"/>
@@ -3486,8 +3658,9 @@
       <c r="N165" s="3"/>
       <c r="O165" s="3"/>
       <c r="P165" s="3"/>
-    </row>
-    <row r="166" spans="1:16">
+      <c r="Q165" s="3"/>
+    </row>
+    <row r="166" spans="1:17">
       <c r="A166" s="3"/>
       <c r="B166" s="3"/>
       <c r="C166" s="3"/>
@@ -3504,8 +3677,9 @@
       <c r="N166" s="3"/>
       <c r="O166" s="3"/>
       <c r="P166" s="3"/>
-    </row>
-    <row r="167" spans="1:16">
+      <c r="Q166" s="3"/>
+    </row>
+    <row r="167" spans="1:17">
       <c r="A167" s="3"/>
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
@@ -3522,8 +3696,9 @@
       <c r="N167" s="3"/>
       <c r="O167" s="3"/>
       <c r="P167" s="3"/>
-    </row>
-    <row r="168" spans="1:16">
+      <c r="Q167" s="3"/>
+    </row>
+    <row r="168" spans="1:17">
       <c r="A168" s="3"/>
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
@@ -3540,8 +3715,9 @@
       <c r="N168" s="3"/>
       <c r="O168" s="3"/>
       <c r="P168" s="3"/>
-    </row>
-    <row r="169" spans="1:16">
+      <c r="Q168" s="3"/>
+    </row>
+    <row r="169" spans="1:17">
       <c r="A169" s="3"/>
       <c r="B169" s="3"/>
       <c r="C169" s="3"/>
@@ -3558,8 +3734,9 @@
       <c r="N169" s="3"/>
       <c r="O169" s="3"/>
       <c r="P169" s="3"/>
-    </row>
-    <row r="170" spans="1:16">
+      <c r="Q169" s="3"/>
+    </row>
+    <row r="170" spans="1:17">
       <c r="A170" s="3"/>
       <c r="B170" s="3"/>
       <c r="C170" s="3"/>
@@ -3576,8 +3753,9 @@
       <c r="N170" s="3"/>
       <c r="O170" s="3"/>
       <c r="P170" s="3"/>
-    </row>
-    <row r="171" spans="1:16">
+      <c r="Q170" s="3"/>
+    </row>
+    <row r="171" spans="1:17">
       <c r="A171" s="3"/>
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
@@ -3594,8 +3772,9 @@
       <c r="N171" s="3"/>
       <c r="O171" s="3"/>
       <c r="P171" s="3"/>
-    </row>
-    <row r="172" spans="1:16">
+      <c r="Q171" s="3"/>
+    </row>
+    <row r="172" spans="1:17">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
@@ -3612,8 +3791,9 @@
       <c r="N172" s="3"/>
       <c r="O172" s="3"/>
       <c r="P172" s="3"/>
-    </row>
-    <row r="173" spans="1:16">
+      <c r="Q172" s="3"/>
+    </row>
+    <row r="173" spans="1:17">
       <c r="A173" s="3"/>
       <c r="B173" s="3"/>
       <c r="C173" s="3"/>
@@ -3630,8 +3810,9 @@
       <c r="N173" s="3"/>
       <c r="O173" s="3"/>
       <c r="P173" s="3"/>
-    </row>
-    <row r="174" spans="1:16">
+      <c r="Q173" s="3"/>
+    </row>
+    <row r="174" spans="1:17">
       <c r="A174" s="3"/>
       <c r="B174" s="3"/>
       <c r="C174" s="3"/>
@@ -3648,8 +3829,9 @@
       <c r="N174" s="3"/>
       <c r="O174" s="3"/>
       <c r="P174" s="3"/>
-    </row>
-    <row r="175" spans="1:16">
+      <c r="Q174" s="3"/>
+    </row>
+    <row r="175" spans="1:17">
       <c r="A175" s="3"/>
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
@@ -3666,8 +3848,9 @@
       <c r="N175" s="3"/>
       <c r="O175" s="3"/>
       <c r="P175" s="3"/>
-    </row>
-    <row r="176" spans="1:16">
+      <c r="Q175" s="3"/>
+    </row>
+    <row r="176" spans="1:17">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
@@ -3684,8 +3867,9 @@
       <c r="N176" s="3"/>
       <c r="O176" s="3"/>
       <c r="P176" s="3"/>
-    </row>
-    <row r="177" spans="1:16">
+      <c r="Q176" s="3"/>
+    </row>
+    <row r="177" spans="1:17">
       <c r="A177" s="3"/>
       <c r="B177" s="3"/>
       <c r="C177" s="3"/>
@@ -3702,8 +3886,9 @@
       <c r="N177" s="3"/>
       <c r="O177" s="3"/>
       <c r="P177" s="3"/>
-    </row>
-    <row r="178" spans="1:16">
+      <c r="Q177" s="3"/>
+    </row>
+    <row r="178" spans="1:17">
       <c r="A178" s="3"/>
       <c r="B178" s="3"/>
       <c r="C178" s="3"/>
@@ -3720,8 +3905,9 @@
       <c r="N178" s="3"/>
       <c r="O178" s="3"/>
       <c r="P178" s="3"/>
-    </row>
-    <row r="179" spans="1:16">
+      <c r="Q178" s="3"/>
+    </row>
+    <row r="179" spans="1:17">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
@@ -3738,8 +3924,9 @@
       <c r="N179" s="3"/>
       <c r="O179" s="3"/>
       <c r="P179" s="3"/>
-    </row>
-    <row r="180" spans="1:16">
+      <c r="Q179" s="3"/>
+    </row>
+    <row r="180" spans="1:17">
       <c r="A180" s="3"/>
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
@@ -3756,8 +3943,9 @@
       <c r="N180" s="3"/>
       <c r="O180" s="3"/>
       <c r="P180" s="3"/>
-    </row>
-    <row r="181" spans="1:16">
+      <c r="Q180" s="3"/>
+    </row>
+    <row r="181" spans="1:17">
       <c r="A181" s="3"/>
       <c r="B181" s="3"/>
       <c r="C181" s="3"/>
@@ -3774,8 +3962,9 @@
       <c r="N181" s="3"/>
       <c r="O181" s="3"/>
       <c r="P181" s="3"/>
-    </row>
-    <row r="182" spans="1:16">
+      <c r="Q181" s="3"/>
+    </row>
+    <row r="182" spans="1:17">
       <c r="A182" s="3"/>
       <c r="B182" s="3"/>
       <c r="C182" s="3"/>
@@ -3792,8 +3981,9 @@
       <c r="N182" s="3"/>
       <c r="O182" s="3"/>
       <c r="P182" s="3"/>
-    </row>
-    <row r="183" spans="1:16">
+      <c r="Q182" s="3"/>
+    </row>
+    <row r="183" spans="1:17">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
@@ -3810,8 +4000,9 @@
       <c r="N183" s="3"/>
       <c r="O183" s="3"/>
       <c r="P183" s="3"/>
-    </row>
-    <row r="184" spans="1:16">
+      <c r="Q183" s="3"/>
+    </row>
+    <row r="184" spans="1:17">
       <c r="A184" s="3"/>
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
@@ -3828,8 +4019,9 @@
       <c r="N184" s="3"/>
       <c r="O184" s="3"/>
       <c r="P184" s="3"/>
-    </row>
-    <row r="185" spans="1:16">
+      <c r="Q184" s="3"/>
+    </row>
+    <row r="185" spans="1:17">
       <c r="A185" s="3"/>
       <c r="B185" s="3"/>
       <c r="C185" s="3"/>
@@ -3846,8 +4038,9 @@
       <c r="N185" s="3"/>
       <c r="O185" s="3"/>
       <c r="P185" s="3"/>
-    </row>
-    <row r="186" spans="1:16">
+      <c r="Q185" s="3"/>
+    </row>
+    <row r="186" spans="1:17">
       <c r="A186" s="3"/>
       <c r="B186" s="3"/>
       <c r="C186" s="3"/>
@@ -3864,8 +4057,9 @@
       <c r="N186" s="3"/>
       <c r="O186" s="3"/>
       <c r="P186" s="3"/>
-    </row>
-    <row r="187" spans="1:16">
+      <c r="Q186" s="3"/>
+    </row>
+    <row r="187" spans="1:17">
       <c r="A187" s="3"/>
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
@@ -3882,8 +4076,9 @@
       <c r="N187" s="3"/>
       <c r="O187" s="3"/>
       <c r="P187" s="3"/>
-    </row>
-    <row r="188" spans="1:16">
+      <c r="Q187" s="3"/>
+    </row>
+    <row r="188" spans="1:17">
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
@@ -3900,8 +4095,9 @@
       <c r="N188" s="3"/>
       <c r="O188" s="3"/>
       <c r="P188" s="3"/>
-    </row>
-    <row r="189" spans="1:16">
+      <c r="Q188" s="3"/>
+    </row>
+    <row r="189" spans="1:17">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
       <c r="C189" s="3"/>
@@ -3918,8 +4114,9 @@
       <c r="N189" s="3"/>
       <c r="O189" s="3"/>
       <c r="P189" s="3"/>
-    </row>
-    <row r="190" spans="1:16">
+      <c r="Q189" s="3"/>
+    </row>
+    <row r="190" spans="1:17">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
       <c r="C190" s="3"/>
@@ -3936,8 +4133,9 @@
       <c r="N190" s="3"/>
       <c r="O190" s="3"/>
       <c r="P190" s="3"/>
-    </row>
-    <row r="191" spans="1:16">
+      <c r="Q190" s="3"/>
+    </row>
+    <row r="191" spans="1:17">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
@@ -3954,8 +4152,9 @@
       <c r="N191" s="3"/>
       <c r="O191" s="3"/>
       <c r="P191" s="3"/>
-    </row>
-    <row r="192" spans="1:16">
+      <c r="Q191" s="3"/>
+    </row>
+    <row r="192" spans="1:17">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
@@ -3972,8 +4171,9 @@
       <c r="N192" s="3"/>
       <c r="O192" s="3"/>
       <c r="P192" s="3"/>
-    </row>
-    <row r="193" spans="1:16">
+      <c r="Q192" s="3"/>
+    </row>
+    <row r="193" spans="1:17">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
       <c r="C193" s="3"/>
@@ -3990,8 +4190,9 @@
       <c r="N193" s="3"/>
       <c r="O193" s="3"/>
       <c r="P193" s="3"/>
-    </row>
-    <row r="194" spans="1:16">
+      <c r="Q193" s="3"/>
+    </row>
+    <row r="194" spans="1:17">
       <c r="A194" s="3"/>
       <c r="B194" s="3"/>
       <c r="C194" s="3"/>
@@ -4008,8 +4209,9 @@
       <c r="N194" s="3"/>
       <c r="O194" s="3"/>
       <c r="P194" s="3"/>
-    </row>
-    <row r="195" spans="1:16">
+      <c r="Q194" s="3"/>
+    </row>
+    <row r="195" spans="1:17">
       <c r="A195" s="3"/>
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
@@ -4026,8 +4228,9 @@
       <c r="N195" s="3"/>
       <c r="O195" s="3"/>
       <c r="P195" s="3"/>
-    </row>
-    <row r="196" spans="1:16">
+      <c r="Q195" s="3"/>
+    </row>
+    <row r="196" spans="1:17">
       <c r="A196" s="3"/>
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
@@ -4044,8 +4247,9 @@
       <c r="N196" s="3"/>
       <c r="O196" s="3"/>
       <c r="P196" s="3"/>
-    </row>
-    <row r="197" spans="1:16">
+      <c r="Q196" s="3"/>
+    </row>
+    <row r="197" spans="1:17">
       <c r="A197" s="3"/>
       <c r="B197" s="3"/>
       <c r="C197" s="3"/>
@@ -4062,8 +4266,9 @@
       <c r="N197" s="3"/>
       <c r="O197" s="3"/>
       <c r="P197" s="3"/>
-    </row>
-    <row r="198" spans="1:16">
+      <c r="Q197" s="3"/>
+    </row>
+    <row r="198" spans="1:17">
       <c r="A198" s="3"/>
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
@@ -4080,8 +4285,9 @@
       <c r="N198" s="3"/>
       <c r="O198" s="3"/>
       <c r="P198" s="3"/>
-    </row>
-    <row r="199" spans="1:16">
+      <c r="Q198" s="3"/>
+    </row>
+    <row r="199" spans="1:17">
       <c r="A199" s="3"/>
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
@@ -4098,8 +4304,9 @@
       <c r="N199" s="3"/>
       <c r="O199" s="3"/>
       <c r="P199" s="3"/>
-    </row>
-    <row r="200" spans="1:16">
+      <c r="Q199" s="3"/>
+    </row>
+    <row r="200" spans="1:17">
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
@@ -4116,8 +4323,9 @@
       <c r="N200" s="3"/>
       <c r="O200" s="3"/>
       <c r="P200" s="3"/>
-    </row>
-    <row r="201" spans="1:16">
+      <c r="Q200" s="3"/>
+    </row>
+    <row r="201" spans="1:17">
       <c r="A201" s="3"/>
       <c r="B201" s="3"/>
       <c r="C201" s="3"/>
@@ -4134,8 +4342,9 @@
       <c r="N201" s="3"/>
       <c r="O201" s="3"/>
       <c r="P201" s="3"/>
-    </row>
-    <row r="202" spans="1:16">
+      <c r="Q201" s="3"/>
+    </row>
+    <row r="202" spans="1:17">
       <c r="A202" s="3"/>
       <c r="B202" s="3"/>
       <c r="C202" s="3"/>
@@ -4152,8 +4361,9 @@
       <c r="N202" s="3"/>
       <c r="O202" s="3"/>
       <c r="P202" s="3"/>
-    </row>
-    <row r="203" spans="1:16">
+      <c r="Q202" s="3"/>
+    </row>
+    <row r="203" spans="1:17">
       <c r="A203" s="3"/>
       <c r="B203" s="3"/>
       <c r="C203" s="3"/>
@@ -4170,8 +4380,9 @@
       <c r="N203" s="3"/>
       <c r="O203" s="3"/>
       <c r="P203" s="3"/>
-    </row>
-    <row r="204" spans="1:16">
+      <c r="Q203" s="3"/>
+    </row>
+    <row r="204" spans="1:17">
       <c r="A204" s="3"/>
       <c r="B204" s="3"/>
       <c r="C204" s="3"/>
@@ -4188,8 +4399,9 @@
       <c r="N204" s="3"/>
       <c r="O204" s="3"/>
       <c r="P204" s="3"/>
-    </row>
-    <row r="205" spans="1:16">
+      <c r="Q204" s="3"/>
+    </row>
+    <row r="205" spans="1:17">
       <c r="A205" s="3"/>
       <c r="B205" s="3"/>
       <c r="C205" s="3"/>
@@ -4206,8 +4418,9 @@
       <c r="N205" s="3"/>
       <c r="O205" s="3"/>
       <c r="P205" s="3"/>
-    </row>
-    <row r="206" spans="1:16">
+      <c r="Q205" s="3"/>
+    </row>
+    <row r="206" spans="1:17">
       <c r="A206" s="3"/>
       <c r="B206" s="3"/>
       <c r="C206" s="3"/>
@@ -4224,8 +4437,9 @@
       <c r="N206" s="3"/>
       <c r="O206" s="3"/>
       <c r="P206" s="3"/>
-    </row>
-    <row r="207" spans="1:16">
+      <c r="Q206" s="3"/>
+    </row>
+    <row r="207" spans="1:17">
       <c r="A207" s="3"/>
       <c r="B207" s="3"/>
       <c r="C207" s="3"/>
@@ -4242,8 +4456,9 @@
       <c r="N207" s="3"/>
       <c r="O207" s="3"/>
       <c r="P207" s="3"/>
-    </row>
-    <row r="208" spans="1:16">
+      <c r="Q207" s="3"/>
+    </row>
+    <row r="208" spans="1:17">
       <c r="A208" s="3"/>
       <c r="B208" s="3"/>
       <c r="C208" s="3"/>
@@ -4260,8 +4475,9 @@
       <c r="N208" s="3"/>
       <c r="O208" s="3"/>
       <c r="P208" s="3"/>
-    </row>
-    <row r="209" spans="1:16">
+      <c r="Q208" s="3"/>
+    </row>
+    <row r="209" spans="1:17">
       <c r="A209" s="3"/>
       <c r="B209" s="3"/>
       <c r="C209" s="3"/>
@@ -4278,8 +4494,9 @@
       <c r="N209" s="3"/>
       <c r="O209" s="3"/>
       <c r="P209" s="3"/>
-    </row>
-    <row r="210" spans="1:16">
+      <c r="Q209" s="3"/>
+    </row>
+    <row r="210" spans="1:17">
       <c r="A210" s="3"/>
       <c r="B210" s="3"/>
       <c r="C210" s="3"/>
@@ -4296,8 +4513,9 @@
       <c r="N210" s="3"/>
       <c r="O210" s="3"/>
       <c r="P210" s="3"/>
-    </row>
-    <row r="211" spans="1:16">
+      <c r="Q210" s="3"/>
+    </row>
+    <row r="211" spans="1:17">
       <c r="A211" s="3"/>
       <c r="B211" s="3"/>
       <c r="C211" s="3"/>
@@ -4314,8 +4532,9 @@
       <c r="N211" s="3"/>
       <c r="O211" s="3"/>
       <c r="P211" s="3"/>
-    </row>
-    <row r="212" spans="1:16">
+      <c r="Q211" s="3"/>
+    </row>
+    <row r="212" spans="1:17">
       <c r="A212" s="3"/>
       <c r="B212" s="3"/>
       <c r="C212" s="3"/>
@@ -4332,8 +4551,9 @@
       <c r="N212" s="3"/>
       <c r="O212" s="3"/>
       <c r="P212" s="3"/>
-    </row>
-    <row r="213" spans="1:16">
+      <c r="Q212" s="3"/>
+    </row>
+    <row r="213" spans="1:17">
       <c r="A213" s="3"/>
       <c r="B213" s="3"/>
       <c r="C213" s="3"/>
@@ -4350,8 +4570,9 @@
       <c r="N213" s="3"/>
       <c r="O213" s="3"/>
       <c r="P213" s="3"/>
-    </row>
-    <row r="214" spans="1:16">
+      <c r="Q213" s="3"/>
+    </row>
+    <row r="214" spans="1:17">
       <c r="A214" s="3"/>
       <c r="B214" s="3"/>
       <c r="C214" s="3"/>
@@ -4368,8 +4589,9 @@
       <c r="N214" s="3"/>
       <c r="O214" s="3"/>
       <c r="P214" s="3"/>
-    </row>
-    <row r="215" spans="1:16">
+      <c r="Q214" s="3"/>
+    </row>
+    <row r="215" spans="1:17">
       <c r="A215" s="3"/>
       <c r="B215" s="3"/>
       <c r="C215" s="3"/>
@@ -4386,8 +4608,9 @@
       <c r="N215" s="3"/>
       <c r="O215" s="3"/>
       <c r="P215" s="3"/>
-    </row>
-    <row r="216" spans="1:16">
+      <c r="Q215" s="3"/>
+    </row>
+    <row r="216" spans="1:17">
       <c r="A216" s="3"/>
       <c r="B216" s="3"/>
       <c r="C216" s="3"/>
@@ -4404,8 +4627,9 @@
       <c r="N216" s="3"/>
       <c r="O216" s="3"/>
       <c r="P216" s="3"/>
-    </row>
-    <row r="217" spans="1:16">
+      <c r="Q216" s="3"/>
+    </row>
+    <row r="217" spans="1:17">
       <c r="A217" s="3"/>
       <c r="B217" s="3"/>
       <c r="C217" s="3"/>
@@ -4422,8 +4646,9 @@
       <c r="N217" s="3"/>
       <c r="O217" s="3"/>
       <c r="P217" s="3"/>
-    </row>
-    <row r="218" spans="1:16">
+      <c r="Q217" s="3"/>
+    </row>
+    <row r="218" spans="1:17">
       <c r="A218" s="3"/>
       <c r="B218" s="3"/>
       <c r="C218" s="3"/>
@@ -4440,8 +4665,9 @@
       <c r="N218" s="3"/>
       <c r="O218" s="3"/>
       <c r="P218" s="3"/>
-    </row>
-    <row r="219" spans="1:16">
+      <c r="Q218" s="3"/>
+    </row>
+    <row r="219" spans="1:17">
       <c r="A219" s="3"/>
       <c r="B219" s="3"/>
       <c r="C219" s="3"/>
@@ -4458,8 +4684,9 @@
       <c r="N219" s="3"/>
       <c r="O219" s="3"/>
       <c r="P219" s="3"/>
-    </row>
-    <row r="220" spans="1:16">
+      <c r="Q219" s="3"/>
+    </row>
+    <row r="220" spans="1:17">
       <c r="A220" s="3"/>
       <c r="B220" s="3"/>
       <c r="C220" s="3"/>
@@ -4476,8 +4703,9 @@
       <c r="N220" s="3"/>
       <c r="O220" s="3"/>
       <c r="P220" s="3"/>
-    </row>
-    <row r="221" spans="1:16">
+      <c r="Q220" s="3"/>
+    </row>
+    <row r="221" spans="1:17">
       <c r="A221" s="3"/>
       <c r="B221" s="3"/>
       <c r="C221" s="3"/>
@@ -4494,8 +4722,9 @@
       <c r="N221" s="3"/>
       <c r="O221" s="3"/>
       <c r="P221" s="3"/>
-    </row>
-    <row r="222" spans="1:16">
+      <c r="Q221" s="3"/>
+    </row>
+    <row r="222" spans="1:17">
       <c r="A222" s="3"/>
       <c r="B222" s="3"/>
       <c r="C222" s="3"/>
@@ -4512,8 +4741,9 @@
       <c r="N222" s="3"/>
       <c r="O222" s="3"/>
       <c r="P222" s="3"/>
-    </row>
-    <row r="223" spans="1:16">
+      <c r="Q222" s="3"/>
+    </row>
+    <row r="223" spans="1:17">
       <c r="A223" s="3"/>
       <c r="B223" s="3"/>
       <c r="C223" s="3"/>
@@ -4530,8 +4760,9 @@
       <c r="N223" s="3"/>
       <c r="O223" s="3"/>
       <c r="P223" s="3"/>
-    </row>
-    <row r="224" spans="1:16">
+      <c r="Q223" s="3"/>
+    </row>
+    <row r="224" spans="1:17">
       <c r="A224" s="3"/>
       <c r="B224" s="3"/>
       <c r="C224" s="3"/>
@@ -4548,8 +4779,9 @@
       <c r="N224" s="3"/>
       <c r="O224" s="3"/>
       <c r="P224" s="3"/>
-    </row>
-    <row r="225" spans="1:16">
+      <c r="Q224" s="3"/>
+    </row>
+    <row r="225" spans="1:17">
       <c r="A225" s="3"/>
       <c r="B225" s="3"/>
       <c r="C225" s="3"/>
@@ -4566,8 +4798,9 @@
       <c r="N225" s="3"/>
       <c r="O225" s="3"/>
       <c r="P225" s="3"/>
-    </row>
-    <row r="226" spans="1:16">
+      <c r="Q225" s="3"/>
+    </row>
+    <row r="226" spans="1:17">
       <c r="A226" s="3"/>
       <c r="B226" s="3"/>
       <c r="C226" s="3"/>
@@ -4584,8 +4817,9 @@
       <c r="N226" s="3"/>
       <c r="O226" s="3"/>
       <c r="P226" s="3"/>
-    </row>
-    <row r="227" spans="1:16">
+      <c r="Q226" s="3"/>
+    </row>
+    <row r="227" spans="1:17">
       <c r="A227" s="3"/>
       <c r="B227" s="3"/>
       <c r="C227" s="3"/>
@@ -4602,8 +4836,9 @@
       <c r="N227" s="3"/>
       <c r="O227" s="3"/>
       <c r="P227" s="3"/>
-    </row>
-    <row r="228" spans="1:16">
+      <c r="Q227" s="3"/>
+    </row>
+    <row r="228" spans="1:17">
       <c r="A228" s="3"/>
       <c r="B228" s="3"/>
       <c r="C228" s="3"/>
@@ -4620,8 +4855,9 @@
       <c r="N228" s="3"/>
       <c r="O228" s="3"/>
       <c r="P228" s="3"/>
-    </row>
-    <row r="229" spans="1:16">
+      <c r="Q228" s="3"/>
+    </row>
+    <row r="229" spans="1:17">
       <c r="A229" s="3"/>
       <c r="B229" s="3"/>
       <c r="C229" s="3"/>
@@ -4638,8 +4874,9 @@
       <c r="N229" s="3"/>
       <c r="O229" s="3"/>
       <c r="P229" s="3"/>
-    </row>
-    <row r="230" spans="1:16">
+      <c r="Q229" s="3"/>
+    </row>
+    <row r="230" spans="1:17">
       <c r="A230" s="3"/>
       <c r="B230" s="3"/>
       <c r="C230" s="3"/>
@@ -4656,8 +4893,9 @@
       <c r="N230" s="3"/>
       <c r="O230" s="3"/>
       <c r="P230" s="3"/>
-    </row>
-    <row r="231" spans="1:16">
+      <c r="Q230" s="3"/>
+    </row>
+    <row r="231" spans="1:17">
       <c r="A231" s="3"/>
       <c r="B231" s="3"/>
       <c r="C231" s="3"/>
@@ -4674,8 +4912,9 @@
       <c r="N231" s="3"/>
       <c r="O231" s="3"/>
       <c r="P231" s="3"/>
-    </row>
-    <row r="232" spans="1:16">
+      <c r="Q231" s="3"/>
+    </row>
+    <row r="232" spans="1:17">
       <c r="A232" s="3"/>
       <c r="B232" s="3"/>
       <c r="C232" s="3"/>
@@ -4692,8 +4931,9 @@
       <c r="N232" s="3"/>
       <c r="O232" s="3"/>
       <c r="P232" s="3"/>
-    </row>
-    <row r="233" spans="1:16">
+      <c r="Q232" s="3"/>
+    </row>
+    <row r="233" spans="1:17">
       <c r="A233" s="3"/>
       <c r="B233" s="3"/>
       <c r="C233" s="3"/>
@@ -4710,8 +4950,9 @@
       <c r="N233" s="3"/>
       <c r="O233" s="3"/>
       <c r="P233" s="3"/>
-    </row>
-    <row r="234" spans="1:16">
+      <c r="Q233" s="3"/>
+    </row>
+    <row r="234" spans="1:17">
       <c r="A234" s="3"/>
       <c r="B234" s="3"/>
       <c r="C234" s="3"/>
@@ -4728,8 +4969,9 @@
       <c r="N234" s="3"/>
       <c r="O234" s="3"/>
       <c r="P234" s="3"/>
-    </row>
-    <row r="235" spans="1:16">
+      <c r="Q234" s="3"/>
+    </row>
+    <row r="235" spans="1:17">
       <c r="A235" s="3"/>
       <c r="B235" s="3"/>
       <c r="C235" s="3"/>
@@ -4746,8 +4988,9 @@
       <c r="N235" s="3"/>
       <c r="O235" s="3"/>
       <c r="P235" s="3"/>
-    </row>
-    <row r="236" spans="1:16">
+      <c r="Q235" s="3"/>
+    </row>
+    <row r="236" spans="1:17">
       <c r="A236" s="3"/>
       <c r="B236" s="3"/>
       <c r="C236" s="3"/>
@@ -4764,8 +5007,9 @@
       <c r="N236" s="3"/>
       <c r="O236" s="3"/>
       <c r="P236" s="3"/>
-    </row>
-    <row r="237" spans="1:16">
+      <c r="Q236" s="3"/>
+    </row>
+    <row r="237" spans="1:17">
       <c r="A237" s="3"/>
       <c r="B237" s="3"/>
       <c r="C237" s="3"/>
@@ -4782,8 +5026,9 @@
       <c r="N237" s="3"/>
       <c r="O237" s="3"/>
       <c r="P237" s="3"/>
-    </row>
-    <row r="238" spans="1:16">
+      <c r="Q237" s="3"/>
+    </row>
+    <row r="238" spans="1:17">
       <c r="A238" s="3"/>
       <c r="B238" s="3"/>
       <c r="C238" s="3"/>
@@ -4800,8 +5045,9 @@
       <c r="N238" s="3"/>
       <c r="O238" s="3"/>
       <c r="P238" s="3"/>
-    </row>
-    <row r="239" spans="1:16">
+      <c r="Q238" s="3"/>
+    </row>
+    <row r="239" spans="1:17">
       <c r="A239" s="3"/>
       <c r="B239" s="3"/>
       <c r="C239" s="3"/>
@@ -4818,8 +5064,9 @@
       <c r="N239" s="3"/>
       <c r="O239" s="3"/>
       <c r="P239" s="3"/>
-    </row>
-    <row r="240" spans="1:16">
+      <c r="Q239" s="3"/>
+    </row>
+    <row r="240" spans="1:17">
       <c r="A240" s="3"/>
       <c r="B240" s="3"/>
       <c r="C240" s="3"/>
@@ -4836,8 +5083,9 @@
       <c r="N240" s="3"/>
       <c r="O240" s="3"/>
       <c r="P240" s="3"/>
-    </row>
-    <row r="241" spans="1:16">
+      <c r="Q240" s="3"/>
+    </row>
+    <row r="241" spans="1:17">
       <c r="A241" s="3"/>
       <c r="B241" s="3"/>
       <c r="C241" s="3"/>
@@ -4854,8 +5102,9 @@
       <c r="N241" s="3"/>
       <c r="O241" s="3"/>
       <c r="P241" s="3"/>
-    </row>
-    <row r="242" spans="1:16">
+      <c r="Q241" s="3"/>
+    </row>
+    <row r="242" spans="1:17">
       <c r="A242" s="3"/>
       <c r="B242" s="3"/>
       <c r="C242" s="3"/>
@@ -4872,8 +5121,9 @@
       <c r="N242" s="3"/>
       <c r="O242" s="3"/>
       <c r="P242" s="3"/>
-    </row>
-    <row r="243" spans="1:16">
+      <c r="Q242" s="3"/>
+    </row>
+    <row r="243" spans="1:17">
       <c r="A243" s="3"/>
       <c r="B243" s="3"/>
       <c r="C243" s="3"/>
@@ -4890,8 +5140,9 @@
       <c r="N243" s="3"/>
       <c r="O243" s="3"/>
       <c r="P243" s="3"/>
-    </row>
-    <row r="244" spans="1:16">
+      <c r="Q243" s="3"/>
+    </row>
+    <row r="244" spans="1:17">
       <c r="A244" s="3"/>
       <c r="B244" s="3"/>
       <c r="C244" s="3"/>
@@ -4908,8 +5159,9 @@
       <c r="N244" s="3"/>
       <c r="O244" s="3"/>
       <c r="P244" s="3"/>
-    </row>
-    <row r="245" spans="1:16">
+      <c r="Q244" s="3"/>
+    </row>
+    <row r="245" spans="1:17">
       <c r="A245" s="3"/>
       <c r="B245" s="3"/>
       <c r="C245" s="3"/>
@@ -4926,8 +5178,9 @@
       <c r="N245" s="3"/>
       <c r="O245" s="3"/>
       <c r="P245" s="3"/>
-    </row>
-    <row r="246" spans="1:16">
+      <c r="Q245" s="3"/>
+    </row>
+    <row r="246" spans="1:17">
       <c r="A246" s="3"/>
       <c r="B246" s="3"/>
       <c r="C246" s="3"/>
@@ -4944,8 +5197,9 @@
       <c r="N246" s="3"/>
       <c r="O246" s="3"/>
       <c r="P246" s="3"/>
-    </row>
-    <row r="247" spans="1:16">
+      <c r="Q246" s="3"/>
+    </row>
+    <row r="247" spans="1:17">
       <c r="A247" s="3"/>
       <c r="B247" s="3"/>
       <c r="C247" s="3"/>
@@ -4962,8 +5216,9 @@
       <c r="N247" s="3"/>
       <c r="O247" s="3"/>
       <c r="P247" s="3"/>
-    </row>
-    <row r="248" spans="1:16">
+      <c r="Q247" s="3"/>
+    </row>
+    <row r="248" spans="1:17">
       <c r="A248" s="3"/>
       <c r="B248" s="3"/>
       <c r="C248" s="3"/>
@@ -4980,8 +5235,9 @@
       <c r="N248" s="3"/>
       <c r="O248" s="3"/>
       <c r="P248" s="3"/>
-    </row>
-    <row r="249" spans="1:16">
+      <c r="Q248" s="3"/>
+    </row>
+    <row r="249" spans="1:17">
       <c r="A249" s="3"/>
       <c r="B249" s="3"/>
       <c r="C249" s="3"/>
@@ -4998,8 +5254,9 @@
       <c r="N249" s="3"/>
       <c r="O249" s="3"/>
       <c r="P249" s="3"/>
-    </row>
-    <row r="250" spans="1:16">
+      <c r="Q249" s="3"/>
+    </row>
+    <row r="250" spans="1:17">
       <c r="A250" s="3"/>
       <c r="B250" s="3"/>
       <c r="C250" s="3"/>
@@ -5016,8 +5273,9 @@
       <c r="N250" s="3"/>
       <c r="O250" s="3"/>
       <c r="P250" s="3"/>
-    </row>
-    <row r="251" spans="1:16">
+      <c r="Q250" s="3"/>
+    </row>
+    <row r="251" spans="1:17">
       <c r="A251" s="3"/>
       <c r="B251" s="3"/>
       <c r="C251" s="3"/>
@@ -5034,8 +5292,9 @@
       <c r="N251" s="3"/>
       <c r="O251" s="3"/>
       <c r="P251" s="3"/>
-    </row>
-    <row r="252" spans="1:16">
+      <c r="Q251" s="3"/>
+    </row>
+    <row r="252" spans="1:17">
       <c r="A252" s="3"/>
       <c r="B252" s="3"/>
       <c r="C252" s="3"/>
@@ -5052,8 +5311,9 @@
       <c r="N252" s="3"/>
       <c r="O252" s="3"/>
       <c r="P252" s="3"/>
-    </row>
-    <row r="253" spans="1:16">
+      <c r="Q252" s="3"/>
+    </row>
+    <row r="253" spans="1:17">
       <c r="A253" s="3"/>
       <c r="B253" s="3"/>
       <c r="C253" s="3"/>
@@ -5070,8 +5330,9 @@
       <c r="N253" s="3"/>
       <c r="O253" s="3"/>
       <c r="P253" s="3"/>
-    </row>
-    <row r="254" spans="1:16">
+      <c r="Q253" s="3"/>
+    </row>
+    <row r="254" spans="1:17">
       <c r="A254" s="3"/>
       <c r="B254" s="3"/>
       <c r="C254" s="3"/>
@@ -5088,8 +5349,9 @@
       <c r="N254" s="3"/>
       <c r="O254" s="3"/>
       <c r="P254" s="3"/>
-    </row>
-    <row r="255" spans="1:16">
+      <c r="Q254" s="3"/>
+    </row>
+    <row r="255" spans="1:17">
       <c r="A255" s="3"/>
       <c r="B255" s="3"/>
       <c r="C255" s="3"/>
@@ -5106,8 +5368,9 @@
       <c r="N255" s="3"/>
       <c r="O255" s="3"/>
       <c r="P255" s="3"/>
-    </row>
-    <row r="256" spans="1:16">
+      <c r="Q255" s="3"/>
+    </row>
+    <row r="256" spans="1:17">
       <c r="A256" s="3"/>
       <c r="B256" s="3"/>
       <c r="C256" s="3"/>
@@ -5124,8 +5387,9 @@
       <c r="N256" s="3"/>
       <c r="O256" s="3"/>
       <c r="P256" s="3"/>
-    </row>
-    <row r="257" spans="1:16">
+      <c r="Q256" s="3"/>
+    </row>
+    <row r="257" spans="1:17">
       <c r="A257" s="3"/>
       <c r="B257" s="3"/>
       <c r="C257" s="3"/>
@@ -5142,8 +5406,9 @@
       <c r="N257" s="3"/>
       <c r="O257" s="3"/>
       <c r="P257" s="3"/>
-    </row>
-    <row r="258" spans="1:16">
+      <c r="Q257" s="3"/>
+    </row>
+    <row r="258" spans="1:17">
       <c r="A258" s="3"/>
       <c r="B258" s="3"/>
       <c r="C258" s="3"/>
@@ -5160,8 +5425,9 @@
       <c r="N258" s="3"/>
       <c r="O258" s="3"/>
       <c r="P258" s="3"/>
-    </row>
-    <row r="259" spans="1:16">
+      <c r="Q258" s="3"/>
+    </row>
+    <row r="259" spans="1:17">
       <c r="A259" s="3"/>
       <c r="B259" s="3"/>
       <c r="C259" s="3"/>
@@ -5178,8 +5444,9 @@
       <c r="N259" s="3"/>
       <c r="O259" s="3"/>
       <c r="P259" s="3"/>
-    </row>
-    <row r="260" spans="1:16">
+      <c r="Q259" s="3"/>
+    </row>
+    <row r="260" spans="1:17">
       <c r="A260" s="3"/>
       <c r="B260" s="3"/>
       <c r="C260" s="3"/>
@@ -5196,8 +5463,9 @@
       <c r="N260" s="3"/>
       <c r="O260" s="3"/>
       <c r="P260" s="3"/>
-    </row>
-    <row r="261" spans="1:16">
+      <c r="Q260" s="3"/>
+    </row>
+    <row r="261" spans="1:17">
       <c r="A261" s="3"/>
       <c r="B261" s="3"/>
       <c r="C261" s="3"/>
@@ -5214,8 +5482,9 @@
       <c r="N261" s="3"/>
       <c r="O261" s="3"/>
       <c r="P261" s="3"/>
-    </row>
-    <row r="262" spans="1:16">
+      <c r="Q261" s="3"/>
+    </row>
+    <row r="262" spans="1:17">
       <c r="A262" s="3"/>
       <c r="B262" s="3"/>
       <c r="C262" s="3"/>
@@ -5232,8 +5501,9 @@
       <c r="N262" s="3"/>
       <c r="O262" s="3"/>
       <c r="P262" s="3"/>
-    </row>
-    <row r="263" spans="1:16">
+      <c r="Q262" s="3"/>
+    </row>
+    <row r="263" spans="1:17">
       <c r="A263" s="3"/>
       <c r="B263" s="3"/>
       <c r="C263" s="3"/>
@@ -5250,8 +5520,9 @@
       <c r="N263" s="3"/>
       <c r="O263" s="3"/>
       <c r="P263" s="3"/>
-    </row>
-    <row r="264" spans="1:16">
+      <c r="Q263" s="3"/>
+    </row>
+    <row r="264" spans="1:17">
       <c r="A264" s="3"/>
       <c r="B264" s="3"/>
       <c r="C264" s="3"/>
@@ -5268,8 +5539,9 @@
       <c r="N264" s="3"/>
       <c r="O264" s="3"/>
       <c r="P264" s="3"/>
-    </row>
-    <row r="265" spans="1:16">
+      <c r="Q264" s="3"/>
+    </row>
+    <row r="265" spans="1:17">
       <c r="A265" s="3"/>
       <c r="B265" s="3"/>
       <c r="C265" s="3"/>
@@ -5286,8 +5558,9 @@
       <c r="N265" s="3"/>
       <c r="O265" s="3"/>
       <c r="P265" s="3"/>
-    </row>
-    <row r="266" spans="1:16">
+      <c r="Q265" s="3"/>
+    </row>
+    <row r="266" spans="1:17">
       <c r="A266" s="3"/>
       <c r="B266" s="3"/>
       <c r="C266" s="3"/>
@@ -5304,8 +5577,9 @@
       <c r="N266" s="3"/>
       <c r="O266" s="3"/>
       <c r="P266" s="3"/>
-    </row>
-    <row r="267" spans="1:16">
+      <c r="Q266" s="3"/>
+    </row>
+    <row r="267" spans="1:17">
       <c r="A267" s="3"/>
       <c r="B267" s="3"/>
       <c r="C267" s="3"/>
@@ -5322,8 +5596,9 @@
       <c r="N267" s="3"/>
       <c r="O267" s="3"/>
       <c r="P267" s="3"/>
-    </row>
-    <row r="268" spans="1:16">
+      <c r="Q267" s="3"/>
+    </row>
+    <row r="268" spans="1:17">
       <c r="A268" s="3"/>
       <c r="B268" s="3"/>
       <c r="C268" s="3"/>
@@ -5340,8 +5615,9 @@
       <c r="N268" s="3"/>
       <c r="O268" s="3"/>
       <c r="P268" s="3"/>
-    </row>
-    <row r="269" spans="1:16">
+      <c r="Q268" s="3"/>
+    </row>
+    <row r="269" spans="1:17">
       <c r="A269" s="3"/>
       <c r="B269" s="3"/>
       <c r="C269" s="3"/>
@@ -5358,8 +5634,9 @@
       <c r="N269" s="3"/>
       <c r="O269" s="3"/>
       <c r="P269" s="3"/>
-    </row>
-    <row r="270" spans="1:16">
+      <c r="Q269" s="3"/>
+    </row>
+    <row r="270" spans="1:17">
       <c r="A270" s="3"/>
       <c r="B270" s="3"/>
       <c r="C270" s="3"/>
@@ -5376,8 +5653,9 @@
       <c r="N270" s="3"/>
       <c r="O270" s="3"/>
       <c r="P270" s="3"/>
-    </row>
-    <row r="271" spans="1:16">
+      <c r="Q270" s="3"/>
+    </row>
+    <row r="271" spans="1:17">
       <c r="A271" s="3"/>
       <c r="B271" s="3"/>
       <c r="C271" s="3"/>
@@ -5394,8 +5672,9 @@
       <c r="N271" s="3"/>
       <c r="O271" s="3"/>
       <c r="P271" s="3"/>
-    </row>
-    <row r="272" spans="1:16">
+      <c r="Q271" s="3"/>
+    </row>
+    <row r="272" spans="1:17">
       <c r="A272" s="3"/>
       <c r="B272" s="3"/>
       <c r="C272" s="3"/>
@@ -5412,8 +5691,9 @@
       <c r="N272" s="3"/>
       <c r="O272" s="3"/>
       <c r="P272" s="3"/>
-    </row>
-    <row r="273" spans="1:16">
+      <c r="Q272" s="3"/>
+    </row>
+    <row r="273" spans="1:17">
       <c r="A273" s="3"/>
       <c r="B273" s="3"/>
       <c r="C273" s="3"/>
@@ -5430,8 +5710,9 @@
       <c r="N273" s="3"/>
       <c r="O273" s="3"/>
       <c r="P273" s="3"/>
-    </row>
-    <row r="274" spans="1:16">
+      <c r="Q273" s="3"/>
+    </row>
+    <row r="274" spans="1:17">
       <c r="A274" s="3"/>
       <c r="B274" s="3"/>
       <c r="C274" s="3"/>
@@ -5448,8 +5729,9 @@
       <c r="N274" s="3"/>
       <c r="O274" s="3"/>
       <c r="P274" s="3"/>
-    </row>
-    <row r="275" spans="1:16">
+      <c r="Q274" s="3"/>
+    </row>
+    <row r="275" spans="1:17">
       <c r="A275" s="3"/>
       <c r="B275" s="3"/>
       <c r="C275" s="3"/>
@@ -5466,8 +5748,9 @@
       <c r="N275" s="3"/>
       <c r="O275" s="3"/>
       <c r="P275" s="3"/>
-    </row>
-    <row r="276" spans="1:16">
+      <c r="Q275" s="3"/>
+    </row>
+    <row r="276" spans="1:17">
       <c r="A276" s="3"/>
       <c r="B276" s="3"/>
       <c r="C276" s="3"/>
@@ -5484,8 +5767,9 @@
       <c r="N276" s="3"/>
       <c r="O276" s="3"/>
       <c r="P276" s="3"/>
-    </row>
-    <row r="277" spans="1:16">
+      <c r="Q276" s="3"/>
+    </row>
+    <row r="277" spans="1:17">
       <c r="A277" s="3"/>
       <c r="B277" s="3"/>
       <c r="C277" s="3"/>
@@ -5502,8 +5786,9 @@
       <c r="N277" s="3"/>
       <c r="O277" s="3"/>
       <c r="P277" s="3"/>
-    </row>
-    <row r="278" spans="1:16">
+      <c r="Q277" s="3"/>
+    </row>
+    <row r="278" spans="1:17">
       <c r="A278" s="3"/>
       <c r="B278" s="3"/>
       <c r="C278" s="3"/>
@@ -5520,8 +5805,9 @@
       <c r="N278" s="3"/>
       <c r="O278" s="3"/>
       <c r="P278" s="3"/>
-    </row>
-    <row r="279" spans="1:16">
+      <c r="Q278" s="3"/>
+    </row>
+    <row r="279" spans="1:17">
       <c r="A279" s="3"/>
       <c r="B279" s="3"/>
       <c r="C279" s="3"/>
@@ -5538,8 +5824,9 @@
       <c r="N279" s="3"/>
       <c r="O279" s="3"/>
       <c r="P279" s="3"/>
-    </row>
-    <row r="280" spans="1:16">
+      <c r="Q279" s="3"/>
+    </row>
+    <row r="280" spans="1:17">
       <c r="A280" s="3"/>
       <c r="B280" s="3"/>
       <c r="C280" s="3"/>
@@ -5556,8 +5843,9 @@
       <c r="N280" s="3"/>
       <c r="O280" s="3"/>
       <c r="P280" s="3"/>
-    </row>
-    <row r="281" spans="1:16">
+      <c r="Q280" s="3"/>
+    </row>
+    <row r="281" spans="1:17">
       <c r="A281" s="3"/>
       <c r="B281" s="3"/>
       <c r="C281" s="3"/>
@@ -5574,8 +5862,9 @@
       <c r="N281" s="3"/>
       <c r="O281" s="3"/>
       <c r="P281" s="3"/>
-    </row>
-    <row r="282" spans="1:16">
+      <c r="Q281" s="3"/>
+    </row>
+    <row r="282" spans="1:17">
       <c r="A282" s="3"/>
       <c r="B282" s="3"/>
       <c r="C282" s="3"/>
@@ -5592,8 +5881,9 @@
       <c r="N282" s="3"/>
       <c r="O282" s="3"/>
       <c r="P282" s="3"/>
-    </row>
-    <row r="283" spans="1:16">
+      <c r="Q282" s="3"/>
+    </row>
+    <row r="283" spans="1:17">
       <c r="A283" s="3"/>
       <c r="B283" s="3"/>
       <c r="C283" s="3"/>
@@ -5610,8 +5900,9 @@
       <c r="N283" s="3"/>
       <c r="O283" s="3"/>
       <c r="P283" s="3"/>
-    </row>
-    <row r="284" spans="1:16">
+      <c r="Q283" s="3"/>
+    </row>
+    <row r="284" spans="1:17">
       <c r="A284" s="3"/>
       <c r="B284" s="3"/>
       <c r="C284" s="3"/>
@@ -5628,8 +5919,9 @@
       <c r="N284" s="3"/>
       <c r="O284" s="3"/>
       <c r="P284" s="3"/>
-    </row>
-    <row r="285" spans="1:16">
+      <c r="Q284" s="3"/>
+    </row>
+    <row r="285" spans="1:17">
       <c r="A285" s="3"/>
       <c r="B285" s="3"/>
       <c r="C285" s="3"/>
@@ -5646,8 +5938,9 @@
       <c r="N285" s="3"/>
       <c r="O285" s="3"/>
       <c r="P285" s="3"/>
-    </row>
-    <row r="286" spans="1:16">
+      <c r="Q285" s="3"/>
+    </row>
+    <row r="286" spans="1:17">
       <c r="A286" s="3"/>
       <c r="B286" s="3"/>
       <c r="C286" s="3"/>
@@ -5664,8 +5957,9 @@
       <c r="N286" s="3"/>
       <c r="O286" s="3"/>
       <c r="P286" s="3"/>
-    </row>
-    <row r="287" spans="1:16">
+      <c r="Q286" s="3"/>
+    </row>
+    <row r="287" spans="1:17">
       <c r="A287" s="3"/>
       <c r="B287" s="3"/>
       <c r="C287" s="3"/>
@@ -5682,8 +5976,9 @@
       <c r="N287" s="3"/>
       <c r="O287" s="3"/>
       <c r="P287" s="3"/>
-    </row>
-    <row r="288" spans="1:16">
+      <c r="Q287" s="3"/>
+    </row>
+    <row r="288" spans="1:17">
       <c r="A288" s="3"/>
       <c r="B288" s="3"/>
       <c r="C288" s="3"/>
@@ -5700,8 +5995,9 @@
       <c r="N288" s="3"/>
       <c r="O288" s="3"/>
       <c r="P288" s="3"/>
-    </row>
-    <row r="289" spans="1:16">
+      <c r="Q288" s="3"/>
+    </row>
+    <row r="289" spans="1:17">
       <c r="A289" s="3"/>
       <c r="B289" s="3"/>
       <c r="C289" s="3"/>
@@ -5718,8 +6014,9 @@
       <c r="N289" s="3"/>
       <c r="O289" s="3"/>
       <c r="P289" s="3"/>
-    </row>
-    <row r="290" spans="1:16">
+      <c r="Q289" s="3"/>
+    </row>
+    <row r="290" spans="1:17">
       <c r="A290" s="3"/>
       <c r="B290" s="3"/>
       <c r="C290" s="3"/>
@@ -5736,8 +6033,9 @@
       <c r="N290" s="3"/>
       <c r="O290" s="3"/>
       <c r="P290" s="3"/>
-    </row>
-    <row r="291" spans="1:16">
+      <c r="Q290" s="3"/>
+    </row>
+    <row r="291" spans="1:17">
       <c r="A291" s="3"/>
       <c r="B291" s="3"/>
       <c r="C291" s="3"/>
@@ -5754,8 +6052,9 @@
       <c r="N291" s="3"/>
       <c r="O291" s="3"/>
       <c r="P291" s="3"/>
-    </row>
-    <row r="292" spans="1:16">
+      <c r="Q291" s="3"/>
+    </row>
+    <row r="292" spans="1:17">
       <c r="A292" s="3"/>
       <c r="B292" s="3"/>
       <c r="C292" s="3"/>
@@ -5772,8 +6071,9 @@
       <c r="N292" s="3"/>
       <c r="O292" s="3"/>
       <c r="P292" s="3"/>
-    </row>
-    <row r="293" spans="1:16">
+      <c r="Q292" s="3"/>
+    </row>
+    <row r="293" spans="1:17">
       <c r="A293" s="3"/>
       <c r="B293" s="3"/>
       <c r="C293" s="3"/>
@@ -5790,8 +6090,9 @@
       <c r="N293" s="3"/>
       <c r="O293" s="3"/>
       <c r="P293" s="3"/>
-    </row>
-    <row r="294" spans="1:16">
+      <c r="Q293" s="3"/>
+    </row>
+    <row r="294" spans="1:17">
       <c r="A294" s="3"/>
       <c r="B294" s="3"/>
       <c r="C294" s="3"/>
@@ -5808,8 +6109,9 @@
       <c r="N294" s="3"/>
       <c r="O294" s="3"/>
       <c r="P294" s="3"/>
-    </row>
-    <row r="295" spans="1:16">
+      <c r="Q294" s="3"/>
+    </row>
+    <row r="295" spans="1:17">
       <c r="A295" s="3"/>
       <c r="B295" s="3"/>
       <c r="C295" s="3"/>
@@ -5826,8 +6128,9 @@
       <c r="N295" s="3"/>
       <c r="O295" s="3"/>
       <c r="P295" s="3"/>
-    </row>
-    <row r="296" spans="1:16">
+      <c r="Q295" s="3"/>
+    </row>
+    <row r="296" spans="1:17">
       <c r="A296" s="3"/>
       <c r="B296" s="3"/>
       <c r="C296" s="3"/>
@@ -5844,8 +6147,9 @@
       <c r="N296" s="3"/>
       <c r="O296" s="3"/>
       <c r="P296" s="3"/>
-    </row>
-    <row r="297" spans="1:16">
+      <c r="Q296" s="3"/>
+    </row>
+    <row r="297" spans="1:17">
       <c r="A297" s="3"/>
       <c r="B297" s="3"/>
       <c r="C297" s="3"/>
@@ -5862,8 +6166,9 @@
       <c r="N297" s="3"/>
       <c r="O297" s="3"/>
       <c r="P297" s="3"/>
-    </row>
-    <row r="298" spans="1:16">
+      <c r="Q297" s="3"/>
+    </row>
+    <row r="298" spans="1:17">
       <c r="A298" s="3"/>
       <c r="B298" s="3"/>
       <c r="C298" s="3"/>
@@ -5880,8 +6185,9 @@
       <c r="N298" s="3"/>
       <c r="O298" s="3"/>
       <c r="P298" s="3"/>
-    </row>
-    <row r="299" spans="1:16">
+      <c r="Q298" s="3"/>
+    </row>
+    <row r="299" spans="1:17">
       <c r="A299" s="3"/>
       <c r="B299" s="3"/>
       <c r="C299" s="3"/>
@@ -5898,8 +6204,9 @@
       <c r="N299" s="3"/>
       <c r="O299" s="3"/>
       <c r="P299" s="3"/>
-    </row>
-    <row r="300" spans="1:16">
+      <c r="Q299" s="3"/>
+    </row>
+    <row r="300" spans="1:17">
       <c r="A300" s="3"/>
       <c r="B300" s="3"/>
       <c r="C300" s="3"/>
@@ -5916,8 +6223,9 @@
       <c r="N300" s="3"/>
       <c r="O300" s="3"/>
       <c r="P300" s="3"/>
-    </row>
-    <row r="301" spans="1:16">
+      <c r="Q300" s="3"/>
+    </row>
+    <row r="301" spans="1:17">
       <c r="A301" s="3"/>
       <c r="B301" s="3"/>
       <c r="C301" s="3"/>
@@ -5934,8 +6242,9 @@
       <c r="N301" s="3"/>
       <c r="O301" s="3"/>
       <c r="P301" s="3"/>
-    </row>
-    <row r="302" spans="1:16">
+      <c r="Q301" s="3"/>
+    </row>
+    <row r="302" spans="1:17">
       <c r="A302" s="3"/>
       <c r="B302" s="3"/>
       <c r="C302" s="3"/>
@@ -5952,8 +6261,9 @@
       <c r="N302" s="3"/>
       <c r="O302" s="3"/>
       <c r="P302" s="3"/>
-    </row>
-    <row r="303" spans="1:16">
+      <c r="Q302" s="3"/>
+    </row>
+    <row r="303" spans="1:17">
       <c r="A303" s="3"/>
       <c r="B303" s="3"/>
       <c r="C303" s="3"/>
@@ -5970,8 +6280,9 @@
       <c r="N303" s="3"/>
       <c r="O303" s="3"/>
       <c r="P303" s="3"/>
-    </row>
-    <row r="304" spans="1:16">
+      <c r="Q303" s="3"/>
+    </row>
+    <row r="304" spans="1:17">
       <c r="A304" s="3"/>
       <c r="B304" s="3"/>
       <c r="C304" s="3"/>
@@ -5988,8 +6299,9 @@
       <c r="N304" s="3"/>
       <c r="O304" s="3"/>
       <c r="P304" s="3"/>
-    </row>
-    <row r="305" spans="1:16">
+      <c r="Q304" s="3"/>
+    </row>
+    <row r="305" spans="1:17">
       <c r="A305" s="3"/>
       <c r="B305" s="3"/>
       <c r="C305" s="3"/>
@@ -6006,8 +6318,9 @@
       <c r="N305" s="3"/>
       <c r="O305" s="3"/>
       <c r="P305" s="3"/>
-    </row>
-    <row r="306" spans="1:16">
+      <c r="Q305" s="3"/>
+    </row>
+    <row r="306" spans="1:17">
       <c r="A306" s="3"/>
       <c r="B306" s="3"/>
       <c r="C306" s="3"/>
@@ -6024,8 +6337,9 @@
       <c r="N306" s="3"/>
       <c r="O306" s="3"/>
       <c r="P306" s="3"/>
-    </row>
-    <row r="307" spans="1:16">
+      <c r="Q306" s="3"/>
+    </row>
+    <row r="307" spans="1:17">
       <c r="A307" s="3"/>
       <c r="B307" s="3"/>
       <c r="C307" s="3"/>
@@ -6042,8 +6356,9 @@
       <c r="N307" s="3"/>
       <c r="O307" s="3"/>
       <c r="P307" s="3"/>
-    </row>
-    <row r="308" spans="1:16">
+      <c r="Q307" s="3"/>
+    </row>
+    <row r="308" spans="1:17">
       <c r="A308" s="3"/>
       <c r="B308" s="3"/>
       <c r="C308" s="3"/>
@@ -6060,8 +6375,9 @@
       <c r="N308" s="3"/>
       <c r="O308" s="3"/>
       <c r="P308" s="3"/>
-    </row>
-    <row r="309" spans="1:16">
+      <c r="Q308" s="3"/>
+    </row>
+    <row r="309" spans="1:17">
       <c r="A309" s="3"/>
       <c r="B309" s="3"/>
       <c r="C309" s="3"/>
@@ -6078,8 +6394,9 @@
       <c r="N309" s="3"/>
       <c r="O309" s="3"/>
       <c r="P309" s="3"/>
-    </row>
-    <row r="310" spans="1:16">
+      <c r="Q309" s="3"/>
+    </row>
+    <row r="310" spans="1:17">
       <c r="A310" s="3"/>
       <c r="B310" s="3"/>
       <c r="C310" s="3"/>
@@ -6096,8 +6413,9 @@
       <c r="N310" s="3"/>
       <c r="O310" s="3"/>
       <c r="P310" s="3"/>
-    </row>
-    <row r="311" spans="1:16">
+      <c r="Q310" s="3"/>
+    </row>
+    <row r="311" spans="1:17">
       <c r="A311" s="3"/>
       <c r="B311" s="3"/>
       <c r="C311" s="3"/>
@@ -6114,8 +6432,9 @@
       <c r="N311" s="3"/>
       <c r="O311" s="3"/>
       <c r="P311" s="3"/>
-    </row>
-    <row r="312" spans="1:16">
+      <c r="Q311" s="3"/>
+    </row>
+    <row r="312" spans="1:17">
       <c r="A312" s="3"/>
       <c r="B312" s="3"/>
       <c r="C312" s="3"/>
@@ -6132,8 +6451,9 @@
       <c r="N312" s="3"/>
       <c r="O312" s="3"/>
       <c r="P312" s="3"/>
-    </row>
-    <row r="313" spans="1:16">
+      <c r="Q312" s="3"/>
+    </row>
+    <row r="313" spans="1:17">
       <c r="A313" s="3"/>
       <c r="B313" s="3"/>
       <c r="C313" s="3"/>
@@ -6150,8 +6470,9 @@
       <c r="N313" s="3"/>
       <c r="O313" s="3"/>
       <c r="P313" s="3"/>
-    </row>
-    <row r="314" spans="1:16">
+      <c r="Q313" s="3"/>
+    </row>
+    <row r="314" spans="1:17">
       <c r="A314" s="3"/>
       <c r="B314" s="3"/>
       <c r="C314" s="3"/>
@@ -6168,8 +6489,9 @@
       <c r="N314" s="3"/>
       <c r="O314" s="3"/>
       <c r="P314" s="3"/>
-    </row>
-    <row r="315" spans="1:16">
+      <c r="Q314" s="3"/>
+    </row>
+    <row r="315" spans="1:17">
       <c r="A315" s="3"/>
       <c r="B315" s="3"/>
       <c r="C315" s="3"/>
@@ -6186,8 +6508,9 @@
       <c r="N315" s="3"/>
       <c r="O315" s="3"/>
       <c r="P315" s="3"/>
-    </row>
-    <row r="316" spans="1:16">
+      <c r="Q315" s="3"/>
+    </row>
+    <row r="316" spans="1:17">
       <c r="A316" s="3"/>
       <c r="B316" s="3"/>
       <c r="C316" s="3"/>
@@ -6204,8 +6527,9 @@
       <c r="N316" s="3"/>
       <c r="O316" s="3"/>
       <c r="P316" s="3"/>
-    </row>
-    <row r="317" spans="1:16">
+      <c r="Q316" s="3"/>
+    </row>
+    <row r="317" spans="1:17">
       <c r="A317" s="3"/>
       <c r="B317" s="3"/>
       <c r="C317" s="3"/>
@@ -6222,8 +6546,9 @@
       <c r="N317" s="3"/>
       <c r="O317" s="3"/>
       <c r="P317" s="3"/>
-    </row>
-    <row r="318" spans="1:16">
+      <c r="Q317" s="3"/>
+    </row>
+    <row r="318" spans="1:17">
       <c r="A318" s="3"/>
       <c r="B318" s="3"/>
       <c r="C318" s="3"/>
@@ -6240,8 +6565,9 @@
       <c r="N318" s="3"/>
       <c r="O318" s="3"/>
       <c r="P318" s="3"/>
-    </row>
-    <row r="319" spans="1:16">
+      <c r="Q318" s="3"/>
+    </row>
+    <row r="319" spans="1:17">
       <c r="A319" s="3"/>
       <c r="B319" s="3"/>
       <c r="C319" s="3"/>
@@ -6258,8 +6584,9 @@
       <c r="N319" s="3"/>
       <c r="O319" s="3"/>
       <c r="P319" s="3"/>
-    </row>
-    <row r="320" spans="1:16">
+      <c r="Q319" s="3"/>
+    </row>
+    <row r="320" spans="1:17">
       <c r="A320" s="3"/>
       <c r="B320" s="3"/>
       <c r="C320" s="3"/>
@@ -6276,8 +6603,9 @@
       <c r="N320" s="3"/>
       <c r="O320" s="3"/>
       <c r="P320" s="3"/>
-    </row>
-    <row r="321" spans="1:16">
+      <c r="Q320" s="3"/>
+    </row>
+    <row r="321" spans="1:17">
       <c r="A321" s="3"/>
       <c r="B321" s="3"/>
       <c r="C321" s="3"/>
@@ -6294,8 +6622,9 @@
       <c r="N321" s="3"/>
       <c r="O321" s="3"/>
       <c r="P321" s="3"/>
-    </row>
-    <row r="322" spans="1:16">
+      <c r="Q321" s="3"/>
+    </row>
+    <row r="322" spans="1:17">
       <c r="A322" s="3"/>
       <c r="B322" s="3"/>
       <c r="C322" s="3"/>
@@ -6312,8 +6641,9 @@
       <c r="N322" s="3"/>
       <c r="O322" s="3"/>
       <c r="P322" s="3"/>
-    </row>
-    <row r="323" spans="1:16">
+      <c r="Q322" s="3"/>
+    </row>
+    <row r="323" spans="1:17">
       <c r="A323" s="3"/>
       <c r="B323" s="3"/>
       <c r="C323" s="3"/>
@@ -6330,8 +6660,9 @@
       <c r="N323" s="3"/>
       <c r="O323" s="3"/>
       <c r="P323" s="3"/>
-    </row>
-    <row r="324" spans="1:16">
+      <c r="Q323" s="3"/>
+    </row>
+    <row r="324" spans="1:17">
       <c r="A324" s="3"/>
       <c r="B324" s="3"/>
       <c r="C324" s="3"/>
@@ -6348,8 +6679,9 @@
       <c r="N324" s="3"/>
       <c r="O324" s="3"/>
       <c r="P324" s="3"/>
-    </row>
-    <row r="325" spans="1:16">
+      <c r="Q324" s="3"/>
+    </row>
+    <row r="325" spans="1:17">
       <c r="A325" s="3"/>
       <c r="B325" s="3"/>
       <c r="C325" s="3"/>
@@ -6366,8 +6698,9 @@
       <c r="N325" s="3"/>
       <c r="O325" s="3"/>
       <c r="P325" s="3"/>
-    </row>
-    <row r="326" spans="1:16">
+      <c r="Q325" s="3"/>
+    </row>
+    <row r="326" spans="1:17">
       <c r="A326" s="3"/>
       <c r="B326" s="3"/>
       <c r="C326" s="3"/>
@@ -6384,8 +6717,9 @@
       <c r="N326" s="3"/>
       <c r="O326" s="3"/>
       <c r="P326" s="3"/>
-    </row>
-    <row r="327" spans="1:16">
+      <c r="Q326" s="3"/>
+    </row>
+    <row r="327" spans="1:17">
       <c r="A327" s="3"/>
       <c r="B327" s="3"/>
       <c r="C327" s="3"/>
@@ -6402,8 +6736,9 @@
       <c r="N327" s="3"/>
       <c r="O327" s="3"/>
       <c r="P327" s="3"/>
-    </row>
-    <row r="328" spans="1:16">
+      <c r="Q327" s="3"/>
+    </row>
+    <row r="328" spans="1:17">
       <c r="A328" s="3"/>
       <c r="B328" s="3"/>
       <c r="C328" s="3"/>
@@ -6420,8 +6755,9 @@
       <c r="N328" s="3"/>
       <c r="O328" s="3"/>
       <c r="P328" s="3"/>
-    </row>
-    <row r="329" spans="1:16">
+      <c r="Q328" s="3"/>
+    </row>
+    <row r="329" spans="1:17">
       <c r="A329" s="3"/>
       <c r="B329" s="3"/>
       <c r="C329" s="3"/>
@@ -6438,8 +6774,9 @@
       <c r="N329" s="3"/>
       <c r="O329" s="3"/>
       <c r="P329" s="3"/>
-    </row>
-    <row r="330" spans="1:16">
+      <c r="Q329" s="3"/>
+    </row>
+    <row r="330" spans="1:17">
       <c r="A330" s="3"/>
       <c r="B330" s="3"/>
       <c r="C330" s="3"/>
@@ -6456,8 +6793,9 @@
       <c r="N330" s="3"/>
       <c r="O330" s="3"/>
       <c r="P330" s="3"/>
-    </row>
-    <row r="331" spans="1:16">
+      <c r="Q330" s="3"/>
+    </row>
+    <row r="331" spans="1:17">
       <c r="A331" s="3"/>
       <c r="B331" s="3"/>
       <c r="C331" s="3"/>
@@ -6474,8 +6812,9 @@
       <c r="N331" s="3"/>
       <c r="O331" s="3"/>
       <c r="P331" s="3"/>
-    </row>
-    <row r="332" spans="1:16">
+      <c r="Q331" s="3"/>
+    </row>
+    <row r="332" spans="1:17">
       <c r="A332" s="3"/>
       <c r="B332" s="3"/>
       <c r="C332" s="3"/>
@@ -6492,8 +6831,9 @@
       <c r="N332" s="3"/>
       <c r="O332" s="3"/>
       <c r="P332" s="3"/>
-    </row>
-    <row r="333" spans="1:16">
+      <c r="Q332" s="3"/>
+    </row>
+    <row r="333" spans="1:17">
       <c r="A333" s="3"/>
       <c r="B333" s="3"/>
       <c r="C333" s="3"/>
@@ -6510,8 +6850,9 @@
       <c r="N333" s="3"/>
       <c r="O333" s="3"/>
       <c r="P333" s="3"/>
-    </row>
-    <row r="334" spans="1:16">
+      <c r="Q333" s="3"/>
+    </row>
+    <row r="334" spans="1:17">
       <c r="A334" s="3"/>
       <c r="B334" s="3"/>
       <c r="C334" s="3"/>
@@ -6528,8 +6869,9 @@
       <c r="N334" s="3"/>
       <c r="O334" s="3"/>
       <c r="P334" s="3"/>
-    </row>
-    <row r="335" spans="1:16">
+      <c r="Q334" s="3"/>
+    </row>
+    <row r="335" spans="1:17">
       <c r="A335" s="3"/>
       <c r="B335" s="3"/>
       <c r="C335" s="3"/>
@@ -6546,8 +6888,9 @@
       <c r="N335" s="3"/>
       <c r="O335" s="3"/>
       <c r="P335" s="3"/>
-    </row>
-    <row r="336" spans="1:16">
+      <c r="Q335" s="3"/>
+    </row>
+    <row r="336" spans="1:17">
       <c r="A336" s="3"/>
       <c r="B336" s="3"/>
       <c r="C336" s="3"/>
@@ -6564,8 +6907,9 @@
       <c r="N336" s="3"/>
       <c r="O336" s="3"/>
       <c r="P336" s="3"/>
-    </row>
-    <row r="337" spans="1:16">
+      <c r="Q336" s="3"/>
+    </row>
+    <row r="337" spans="1:17">
       <c r="A337" s="3"/>
       <c r="B337" s="3"/>
       <c r="C337" s="3"/>
@@ -6582,8 +6926,9 @@
       <c r="N337" s="3"/>
       <c r="O337" s="3"/>
       <c r="P337" s="3"/>
-    </row>
-    <row r="338" spans="1:16">
+      <c r="Q337" s="3"/>
+    </row>
+    <row r="338" spans="1:17">
       <c r="A338" s="3"/>
       <c r="B338" s="3"/>
       <c r="C338" s="3"/>
@@ -6600,8 +6945,9 @@
       <c r="N338" s="3"/>
       <c r="O338" s="3"/>
       <c r="P338" s="3"/>
-    </row>
-    <row r="339" spans="1:16">
+      <c r="Q338" s="3"/>
+    </row>
+    <row r="339" spans="1:17">
       <c r="A339" s="3"/>
       <c r="B339" s="3"/>
       <c r="C339" s="3"/>
@@ -6618,8 +6964,9 @@
       <c r="N339" s="3"/>
       <c r="O339" s="3"/>
       <c r="P339" s="3"/>
-    </row>
-    <row r="340" spans="1:16">
+      <c r="Q339" s="3"/>
+    </row>
+    <row r="340" spans="1:17">
       <c r="A340" s="3"/>
       <c r="B340" s="3"/>
       <c r="C340" s="3"/>
@@ -6636,8 +6983,9 @@
       <c r="N340" s="3"/>
       <c r="O340" s="3"/>
       <c r="P340" s="3"/>
-    </row>
-    <row r="341" spans="1:16">
+      <c r="Q340" s="3"/>
+    </row>
+    <row r="341" spans="1:17">
       <c r="A341" s="3"/>
       <c r="B341" s="3"/>
       <c r="C341" s="3"/>
@@ -6654,8 +7002,9 @@
       <c r="N341" s="3"/>
       <c r="O341" s="3"/>
       <c r="P341" s="3"/>
-    </row>
-    <row r="342" spans="1:16">
+      <c r="Q341" s="3"/>
+    </row>
+    <row r="342" spans="1:17">
       <c r="A342" s="3"/>
       <c r="B342" s="3"/>
       <c r="C342" s="3"/>
@@ -6672,8 +7021,9 @@
       <c r="N342" s="3"/>
       <c r="O342" s="3"/>
       <c r="P342" s="3"/>
-    </row>
-    <row r="343" spans="1:16">
+      <c r="Q342" s="3"/>
+    </row>
+    <row r="343" spans="1:17">
       <c r="A343" s="3"/>
       <c r="B343" s="3"/>
       <c r="C343" s="3"/>
@@ -6690,8 +7040,9 @@
       <c r="N343" s="3"/>
       <c r="O343" s="3"/>
       <c r="P343" s="3"/>
-    </row>
-    <row r="344" spans="1:16">
+      <c r="Q343" s="3"/>
+    </row>
+    <row r="344" spans="1:17">
       <c r="A344" s="3"/>
       <c r="B344" s="3"/>
       <c r="C344" s="3"/>
@@ -6708,8 +7059,9 @@
       <c r="N344" s="3"/>
       <c r="O344" s="3"/>
       <c r="P344" s="3"/>
-    </row>
-    <row r="345" spans="1:16">
+      <c r="Q344" s="3"/>
+    </row>
+    <row r="345" spans="1:17">
       <c r="A345" s="3"/>
       <c r="B345" s="3"/>
       <c r="C345" s="3"/>
@@ -6726,8 +7078,9 @@
       <c r="N345" s="3"/>
       <c r="O345" s="3"/>
       <c r="P345" s="3"/>
-    </row>
-    <row r="346" spans="1:16">
+      <c r="Q345" s="3"/>
+    </row>
+    <row r="346" spans="1:17">
       <c r="A346" s="3"/>
       <c r="B346" s="3"/>
       <c r="C346" s="3"/>
@@ -6744,8 +7097,9 @@
       <c r="N346" s="3"/>
       <c r="O346" s="3"/>
       <c r="P346" s="3"/>
-    </row>
-    <row r="347" spans="1:16">
+      <c r="Q346" s="3"/>
+    </row>
+    <row r="347" spans="1:17">
       <c r="A347" s="3"/>
       <c r="B347" s="3"/>
       <c r="C347" s="3"/>
@@ -6762,8 +7116,9 @@
       <c r="N347" s="3"/>
       <c r="O347" s="3"/>
       <c r="P347" s="3"/>
-    </row>
-    <row r="348" spans="1:16">
+      <c r="Q347" s="3"/>
+    </row>
+    <row r="348" spans="1:17">
       <c r="A348" s="3"/>
       <c r="B348" s="3"/>
       <c r="C348" s="3"/>
@@ -6780,8 +7135,9 @@
       <c r="N348" s="3"/>
       <c r="O348" s="3"/>
       <c r="P348" s="3"/>
-    </row>
-    <row r="349" spans="1:16">
+      <c r="Q348" s="3"/>
+    </row>
+    <row r="349" spans="1:17">
       <c r="A349" s="3"/>
       <c r="B349" s="3"/>
       <c r="C349" s="3"/>
@@ -6798,8 +7154,9 @@
       <c r="N349" s="3"/>
       <c r="O349" s="3"/>
       <c r="P349" s="3"/>
-    </row>
-    <row r="350" spans="1:16">
+      <c r="Q349" s="3"/>
+    </row>
+    <row r="350" spans="1:17">
       <c r="A350" s="3"/>
       <c r="B350" s="3"/>
       <c r="C350" s="3"/>
@@ -6816,8 +7173,9 @@
       <c r="N350" s="3"/>
       <c r="O350" s="3"/>
       <c r="P350" s="3"/>
-    </row>
-    <row r="351" spans="1:16">
+      <c r="Q350" s="3"/>
+    </row>
+    <row r="351" spans="1:17">
       <c r="A351" s="3"/>
       <c r="B351" s="3"/>
       <c r="C351" s="3"/>
@@ -6834,8 +7192,9 @@
       <c r="N351" s="3"/>
       <c r="O351" s="3"/>
       <c r="P351" s="3"/>
-    </row>
-    <row r="352" spans="1:16">
+      <c r="Q351" s="3"/>
+    </row>
+    <row r="352" spans="1:17">
       <c r="A352" s="3"/>
       <c r="B352" s="3"/>
       <c r="C352" s="3"/>
@@ -6852,8 +7211,9 @@
       <c r="N352" s="3"/>
       <c r="O352" s="3"/>
       <c r="P352" s="3"/>
-    </row>
-    <row r="353" spans="1:16">
+      <c r="Q352" s="3"/>
+    </row>
+    <row r="353" spans="1:17">
       <c r="A353" s="3"/>
       <c r="B353" s="3"/>
       <c r="C353" s="3"/>
@@ -6870,8 +7230,9 @@
       <c r="N353" s="3"/>
       <c r="O353" s="3"/>
       <c r="P353" s="3"/>
-    </row>
-    <row r="354" spans="1:16">
+      <c r="Q353" s="3"/>
+    </row>
+    <row r="354" spans="1:17">
       <c r="A354" s="3"/>
       <c r="B354" s="3"/>
       <c r="C354" s="3"/>
@@ -6888,8 +7249,9 @@
       <c r="N354" s="3"/>
       <c r="O354" s="3"/>
       <c r="P354" s="3"/>
-    </row>
-    <row r="355" spans="1:16">
+      <c r="Q354" s="3"/>
+    </row>
+    <row r="355" spans="1:17">
       <c r="A355" s="3"/>
       <c r="B355" s="3"/>
       <c r="C355" s="3"/>
@@ -6906,8 +7268,9 @@
       <c r="N355" s="3"/>
       <c r="O355" s="3"/>
       <c r="P355" s="3"/>
-    </row>
-    <row r="356" spans="1:16">
+      <c r="Q355" s="3"/>
+    </row>
+    <row r="356" spans="1:17">
       <c r="A356" s="3"/>
       <c r="B356" s="3"/>
       <c r="C356" s="3"/>
@@ -6924,8 +7287,9 @@
       <c r="N356" s="3"/>
       <c r="O356" s="3"/>
       <c r="P356" s="3"/>
-    </row>
-    <row r="357" spans="1:16">
+      <c r="Q356" s="3"/>
+    </row>
+    <row r="357" spans="1:17">
       <c r="A357" s="3"/>
       <c r="B357" s="3"/>
       <c r="C357" s="3"/>
@@ -6942,8 +7306,9 @@
       <c r="N357" s="3"/>
       <c r="O357" s="3"/>
       <c r="P357" s="3"/>
-    </row>
-    <row r="358" spans="1:16">
+      <c r="Q357" s="3"/>
+    </row>
+    <row r="358" spans="1:17">
       <c r="A358" s="3"/>
       <c r="B358" s="3"/>
       <c r="C358" s="3"/>
@@ -6960,8 +7325,9 @@
       <c r="N358" s="3"/>
       <c r="O358" s="3"/>
       <c r="P358" s="3"/>
-    </row>
-    <row r="359" spans="1:16">
+      <c r="Q358" s="3"/>
+    </row>
+    <row r="359" spans="1:17">
       <c r="A359" s="3"/>
       <c r="B359" s="3"/>
       <c r="C359" s="3"/>
@@ -6978,8 +7344,9 @@
       <c r="N359" s="3"/>
       <c r="O359" s="3"/>
       <c r="P359" s="3"/>
-    </row>
-    <row r="360" spans="1:16">
+      <c r="Q359" s="3"/>
+    </row>
+    <row r="360" spans="1:17">
       <c r="A360" s="3"/>
       <c r="B360" s="3"/>
       <c r="C360" s="3"/>
@@ -6996,8 +7363,9 @@
       <c r="N360" s="3"/>
       <c r="O360" s="3"/>
       <c r="P360" s="3"/>
-    </row>
-    <row r="361" spans="1:16">
+      <c r="Q360" s="3"/>
+    </row>
+    <row r="361" spans="1:17">
       <c r="A361" s="3"/>
       <c r="B361" s="3"/>
       <c r="C361" s="3"/>
@@ -7014,8 +7382,9 @@
       <c r="N361" s="3"/>
       <c r="O361" s="3"/>
       <c r="P361" s="3"/>
-    </row>
-    <row r="362" spans="1:16">
+      <c r="Q361" s="3"/>
+    </row>
+    <row r="362" spans="1:17">
       <c r="A362" s="3"/>
       <c r="B362" s="3"/>
       <c r="C362" s="3"/>
@@ -7032,8 +7401,9 @@
       <c r="N362" s="3"/>
       <c r="O362" s="3"/>
       <c r="P362" s="3"/>
-    </row>
-    <row r="363" spans="1:16">
+      <c r="Q362" s="3"/>
+    </row>
+    <row r="363" spans="1:17">
       <c r="A363" s="3"/>
       <c r="B363" s="3"/>
       <c r="C363" s="3"/>
@@ -7050,8 +7420,9 @@
       <c r="N363" s="3"/>
       <c r="O363" s="3"/>
       <c r="P363" s="3"/>
-    </row>
-    <row r="364" spans="1:16">
+      <c r="Q363" s="3"/>
+    </row>
+    <row r="364" spans="1:17">
       <c r="A364" s="3"/>
       <c r="B364" s="3"/>
       <c r="C364" s="3"/>
@@ -7068,8 +7439,9 @@
       <c r="N364" s="3"/>
       <c r="O364" s="3"/>
       <c r="P364" s="3"/>
-    </row>
-    <row r="365" spans="1:16">
+      <c r="Q364" s="3"/>
+    </row>
+    <row r="365" spans="1:17">
       <c r="A365" s="3"/>
       <c r="B365" s="3"/>
       <c r="C365" s="3"/>
@@ -7086,8 +7458,9 @@
       <c r="N365" s="3"/>
       <c r="O365" s="3"/>
       <c r="P365" s="3"/>
-    </row>
-    <row r="366" spans="1:16">
+      <c r="Q365" s="3"/>
+    </row>
+    <row r="366" spans="1:17">
       <c r="A366" s="3"/>
       <c r="B366" s="3"/>
       <c r="C366" s="3"/>
@@ -7104,8 +7477,9 @@
       <c r="N366" s="3"/>
       <c r="O366" s="3"/>
       <c r="P366" s="3"/>
-    </row>
-    <row r="367" spans="1:16">
+      <c r="Q366" s="3"/>
+    </row>
+    <row r="367" spans="1:17">
       <c r="A367" s="3"/>
       <c r="B367" s="3"/>
       <c r="C367" s="3"/>
@@ -7122,8 +7496,9 @@
       <c r="N367" s="3"/>
       <c r="O367" s="3"/>
       <c r="P367" s="3"/>
-    </row>
-    <row r="368" spans="1:16">
+      <c r="Q367" s="3"/>
+    </row>
+    <row r="368" spans="1:17">
       <c r="A368" s="3"/>
       <c r="B368" s="3"/>
       <c r="C368" s="3"/>
@@ -7140,8 +7515,9 @@
       <c r="N368" s="3"/>
       <c r="O368" s="3"/>
       <c r="P368" s="3"/>
-    </row>
-    <row r="369" spans="1:16">
+      <c r="Q368" s="3"/>
+    </row>
+    <row r="369" spans="1:17">
       <c r="A369" s="3"/>
       <c r="B369" s="3"/>
       <c r="C369" s="3"/>
@@ -7158,8 +7534,9 @@
       <c r="N369" s="3"/>
       <c r="O369" s="3"/>
       <c r="P369" s="3"/>
-    </row>
-    <row r="370" spans="1:16">
+      <c r="Q369" s="3"/>
+    </row>
+    <row r="370" spans="1:17">
       <c r="A370" s="3"/>
       <c r="B370" s="3"/>
       <c r="C370" s="3"/>
@@ -7176,8 +7553,9 @@
       <c r="N370" s="3"/>
       <c r="O370" s="3"/>
       <c r="P370" s="3"/>
-    </row>
-    <row r="371" spans="1:16">
+      <c r="Q370" s="3"/>
+    </row>
+    <row r="371" spans="1:17">
       <c r="A371" s="3"/>
       <c r="B371" s="3"/>
       <c r="C371" s="3"/>
@@ -7194,8 +7572,9 @@
       <c r="N371" s="3"/>
       <c r="O371" s="3"/>
       <c r="P371" s="3"/>
-    </row>
-    <row r="372" spans="1:16">
+      <c r="Q371" s="3"/>
+    </row>
+    <row r="372" spans="1:17">
       <c r="A372" s="3"/>
       <c r="B372" s="3"/>
       <c r="C372" s="3"/>
@@ -7212,8 +7591,9 @@
       <c r="N372" s="3"/>
       <c r="O372" s="3"/>
       <c r="P372" s="3"/>
-    </row>
-    <row r="373" spans="1:16">
+      <c r="Q372" s="3"/>
+    </row>
+    <row r="373" spans="1:17">
       <c r="A373" s="3"/>
       <c r="B373" s="3"/>
       <c r="C373" s="3"/>
@@ -7230,8 +7610,9 @@
       <c r="N373" s="3"/>
       <c r="O373" s="3"/>
       <c r="P373" s="3"/>
-    </row>
-    <row r="374" spans="1:16">
+      <c r="Q373" s="3"/>
+    </row>
+    <row r="374" spans="1:17">
       <c r="A374" s="3"/>
       <c r="B374" s="3"/>
       <c r="C374" s="3"/>
@@ -7248,8 +7629,9 @@
       <c r="N374" s="3"/>
       <c r="O374" s="3"/>
       <c r="P374" s="3"/>
-    </row>
-    <row r="375" spans="1:16">
+      <c r="Q374" s="3"/>
+    </row>
+    <row r="375" spans="1:17">
       <c r="A375" s="3"/>
       <c r="B375" s="3"/>
       <c r="C375" s="3"/>
@@ -7266,6 +7648,7 @@
       <c r="N375" s="3"/>
       <c r="O375" s="3"/>
       <c r="P375" s="3"/>
+      <c r="Q375" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ativa follow-up 48h e 5 dias
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\yamaha-bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B85303FB-6B0D-46E3-B735-EA4ACE85BF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4088344C-E0B1-43F8-BE36-8856003287A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1730,6 +1730,7 @@
     <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Ajuste dashboard crm com itens vendidos
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\yamaha-bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4088344C-E0B1-43F8-BE36-8856003287A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D52FFA00-9005-4011-9107-A646703825D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="310">
   <si>
     <t>NOME</t>
   </si>
@@ -950,417 +950,6 @@
   </si>
   <si>
     <t>9C6RG9920S0021329</t>
-  </si>
-  <si>
-    <t>ROSIMERE MARTINS DOS SANTOS</t>
-  </si>
-  <si>
-    <t>5591980143367</t>
-  </si>
-  <si>
-    <t>9C6RG9910S0043311</t>
-  </si>
-  <si>
-    <t>EDINALDO DOS SANTOS RODRIGUES</t>
-  </si>
-  <si>
-    <t>5594981162830</t>
-  </si>
-  <si>
-    <t>9C6DG25G0S0015360</t>
-  </si>
-  <si>
-    <t>ANDREIA ASSUNCAO DE AVELAR</t>
-  </si>
-  <si>
-    <t>9C6RG7720S0034870</t>
-  </si>
-  <si>
-    <t>JOSE LUCIO FERREIRA DE SOUSA</t>
-  </si>
-  <si>
-    <t>5594992237882</t>
-  </si>
-  <si>
-    <t>9C6DG3340S0033950</t>
-  </si>
-  <si>
-    <t>HENRIQUE BRUNO DA SILVA OLIVEIRA</t>
-  </si>
-  <si>
-    <t>5594992147756</t>
-  </si>
-  <si>
-    <t>9C6RG7720S0035510</t>
-  </si>
-  <si>
-    <t>DILVANI MARINHO FEITOSA</t>
-  </si>
-  <si>
-    <t>5594991621910</t>
-  </si>
-  <si>
-    <t>9C6RG9910S0043366</t>
-  </si>
-  <si>
-    <t>JUCILENE DO NASCIMENTO OLIVEIRA</t>
-  </si>
-  <si>
-    <t>5594999737260</t>
-  </si>
-  <si>
-    <t>9C6RG7720S0034743</t>
-  </si>
-  <si>
-    <t>VITOR GABRIEL ARAUJO DOS SANTOS</t>
-  </si>
-  <si>
-    <t>5594991883219</t>
-  </si>
-  <si>
-    <t>9C6DG3340S0042416</t>
-  </si>
-  <si>
-    <t>JOSIMAR ROCHA SOUSA</t>
-  </si>
-  <si>
-    <t>5594999749991</t>
-  </si>
-  <si>
-    <t>9C6DG3340S0041426</t>
-  </si>
-  <si>
-    <t>AMANDA COELHO SANTOS</t>
-  </si>
-  <si>
-    <t>5591984139295</t>
-  </si>
-  <si>
-    <t>9C6RG7720T0037302</t>
-  </si>
-  <si>
-    <t>MIGUEL ANGELO RODRIGUES MOCBEL</t>
-  </si>
-  <si>
-    <t>5591980867954</t>
-  </si>
-  <si>
-    <t>9C6DG3340S0032569</t>
-  </si>
-  <si>
-    <t>CLEOMAR DOS SANTOS FARIA</t>
-  </si>
-  <si>
-    <t>5594999187832</t>
-  </si>
-  <si>
-    <t>9C6DG3340S0041903</t>
-  </si>
-  <si>
-    <t>9C6RG9910S0044177</t>
-  </si>
-  <si>
-    <t>EDIVANIA DA SILVA SOUSA</t>
-  </si>
-  <si>
-    <t>5599984537061</t>
-  </si>
-  <si>
-    <t>9C6RG9910S0039090</t>
-  </si>
-  <si>
-    <t>MAX JUNIOR PINHEIRO DOS SANTOS</t>
-  </si>
-  <si>
-    <t>5591987070831</t>
-  </si>
-  <si>
-    <t>9C6RG5040S0040945</t>
-  </si>
-  <si>
-    <t>AUGUSTO CESAR PIRES MARINHO</t>
-  </si>
-  <si>
-    <t>5594981122408</t>
-  </si>
-  <si>
-    <t>9C6DG25F0S0019387</t>
-  </si>
-  <si>
-    <t>9C6DG25G0T0021482</t>
-  </si>
-  <si>
-    <t>9C6RG9910T0063163</t>
-  </si>
-  <si>
-    <t>9C6RG9910T0061680</t>
-  </si>
-  <si>
-    <t>POLIANA SILVA SANTOS</t>
-  </si>
-  <si>
-    <t>5594992811365</t>
-  </si>
-  <si>
-    <t>9C6RG8310T0021815</t>
-  </si>
-  <si>
-    <t>MARIA CLARA CARNEIRO DE SOUZA</t>
-  </si>
-  <si>
-    <t>5594999554940</t>
-  </si>
-  <si>
-    <t>9C6DG25F0T0020786</t>
-  </si>
-  <si>
-    <t>SEBASTIAO PEDRO DE OLIVEIRA FILHO</t>
-  </si>
-  <si>
-    <t>5592991413111</t>
-  </si>
-  <si>
-    <t>9C6RG5040T0065581</t>
-  </si>
-  <si>
-    <t>IVANETE DA SILVA ALCANTARA REIS</t>
-  </si>
-  <si>
-    <t>5594996642615</t>
-  </si>
-  <si>
-    <t>9C6RG7720T0050027</t>
-  </si>
-  <si>
-    <t>ALEXANDER BRYAN DE SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>5594992616696</t>
-  </si>
-  <si>
-    <t>9C6RG8310T0021746</t>
-  </si>
-  <si>
-    <t>ABRAAO CABRAL DOS SANTOS NETO</t>
-  </si>
-  <si>
-    <t>5594988063592</t>
-  </si>
-  <si>
-    <t>9C6DG3340T0053833</t>
-  </si>
-  <si>
-    <t>GILMAR ALVES DE PAULA</t>
-  </si>
-  <si>
-    <t>5594981704501</t>
-  </si>
-  <si>
-    <t>9C6SEK910V0017308</t>
-  </si>
-  <si>
-    <t>FLUO VERSAO 125 HYBRID</t>
-  </si>
-  <si>
-    <t>VALQUIRIA DA SILVA ALVES</t>
-  </si>
-  <si>
-    <t>5594992726065</t>
-  </si>
-  <si>
-    <t>9C6RG7720T0049546</t>
-  </si>
-  <si>
-    <t>JONATAS CRUZ DA SILVA</t>
-  </si>
-  <si>
-    <t>5594999730969</t>
-  </si>
-  <si>
-    <t>9C6DG3340S0047834</t>
-  </si>
-  <si>
-    <t>FRANCISCO DAS CHAGAS SANTOS SILVA</t>
-  </si>
-  <si>
-    <t>5594991154814</t>
-  </si>
-  <si>
-    <t>9C6RG8310T0021426</t>
-  </si>
-  <si>
-    <t>BRUNO COELHO DAS NEVES</t>
-  </si>
-  <si>
-    <t>5594991056688</t>
-  </si>
-  <si>
-    <t>9C6DG3340T0053324</t>
-  </si>
-  <si>
-    <t>ILNALDO CHAGAS MELO</t>
-  </si>
-  <si>
-    <t>5594991700470</t>
-  </si>
-  <si>
-    <t>9C6DG25F0S0018516</t>
-  </si>
-  <si>
-    <t>ADRIANO ANDRE DE OLIVEIRA</t>
-  </si>
-  <si>
-    <t>5594988154461</t>
-  </si>
-  <si>
-    <t>9C6DG3340T0050747</t>
-  </si>
-  <si>
-    <t>SALUSTIANO GUITARRA DE SOUZA</t>
-  </si>
-  <si>
-    <t>5594992118232</t>
-  </si>
-  <si>
-    <t>9C6RG7720T0050832</t>
-  </si>
-  <si>
-    <t>ANDERSON DA SILVA GARCIA</t>
-  </si>
-  <si>
-    <t>5594999242109</t>
-  </si>
-  <si>
-    <t>9C6RG5040T0067534</t>
-  </si>
-  <si>
-    <t>GESSICA FERREIRA DA CUNHA</t>
-  </si>
-  <si>
-    <t>5594998123658</t>
-  </si>
-  <si>
-    <t>9C6RG5040T0064166</t>
-  </si>
-  <si>
-    <t>DENILSON SANTOS BORGES</t>
-  </si>
-  <si>
-    <t>5594984007331</t>
-  </si>
-  <si>
-    <t>9C6RG7720T0050658</t>
-  </si>
-  <si>
-    <t>GILLANA COSTA DE MORAES</t>
-  </si>
-  <si>
-    <t>5594996621321</t>
-  </si>
-  <si>
-    <t>9C6RG7720T0049543</t>
-  </si>
-  <si>
-    <t>DAYANE CASTRO DE OLIVEIRA</t>
-  </si>
-  <si>
-    <t>5594992129235</t>
-  </si>
-  <si>
-    <t>9C6RG5040T0065824</t>
-  </si>
-  <si>
-    <t>DARLEISON WANDERSON SILVA PINHEIRO</t>
-  </si>
-  <si>
-    <t>5591981719314</t>
-  </si>
-  <si>
-    <t>9C6RG8310T0021771</t>
-  </si>
-  <si>
-    <t>ALBERTO DA SILVA MOURAO</t>
-  </si>
-  <si>
-    <t>5594991897401</t>
-  </si>
-  <si>
-    <t>9C6DG25F0T0020920</t>
-  </si>
-  <si>
-    <t>BARBARA SILVA DIAS</t>
-  </si>
-  <si>
-    <t>5591993191268</t>
-  </si>
-  <si>
-    <t>9C6RG5040T0065573</t>
-  </si>
-  <si>
-    <t>JACKSON FONTES DA SILVA</t>
-  </si>
-  <si>
-    <t>5531999201627</t>
-  </si>
-  <si>
-    <t>9C6DG3340T0056792</t>
-  </si>
-  <si>
-    <t>FELIPE ALMEIDA PIMENTA</t>
-  </si>
-  <si>
-    <t>5531995868866</t>
-  </si>
-  <si>
-    <t>9C6SGA210T0002020</t>
-  </si>
-  <si>
-    <t>AEROX VERSAO 160</t>
-  </si>
-  <si>
-    <t>MATIAS HENRIQUE LOPES LUCENA</t>
-  </si>
-  <si>
-    <t>5594988074480</t>
-  </si>
-  <si>
-    <t>9C6SGA210T0004283</t>
-  </si>
-  <si>
-    <t>GEDERSON AZEVEDO RIBEIRO</t>
-  </si>
-  <si>
-    <t>5594981507188</t>
-  </si>
-  <si>
-    <t>9C6RG7720T0048246</t>
-  </si>
-  <si>
-    <t>MAGNO ANTONINI DA LUZ MORAES</t>
-  </si>
-  <si>
-    <t>5594991120558</t>
-  </si>
-  <si>
-    <t>9C6RG7720T0051170</t>
-  </si>
-  <si>
-    <t>WEMERSON DOS SANTOS MARTINS</t>
-  </si>
-  <si>
-    <t>5591984405768</t>
-  </si>
-  <si>
-    <t>9C6RG7720T0050030</t>
-  </si>
-  <si>
-    <t>IRACEMA QUEIROZ DE OLIVEIRA</t>
-  </si>
-  <si>
-    <t>5594999344980</t>
-  </si>
-  <si>
-    <t>9C6DG25F0T0020696</t>
   </si>
 </sst>
 </file>
@@ -1724,7 +1313,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q131"/>
+  <dimension ref="A1:Q83"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
@@ -4912,822 +4501,6 @@
         <v>27</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>310</v>
-      </c>
-      <c r="B84" t="s">
-        <v>311</v>
-      </c>
-      <c r="C84" t="s">
-        <v>46</v>
-      </c>
-      <c r="D84" t="s">
-        <v>312</v>
-      </c>
-      <c r="E84" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>313</v>
-      </c>
-      <c r="B85" t="s">
-        <v>314</v>
-      </c>
-      <c r="C85" t="s">
-        <v>19</v>
-      </c>
-      <c r="D85" t="s">
-        <v>315</v>
-      </c>
-      <c r="E85" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
-        <v>316</v>
-      </c>
-      <c r="B86" t="s">
-        <v>75</v>
-      </c>
-      <c r="C86" t="s">
-        <v>19</v>
-      </c>
-      <c r="D86" t="s">
-        <v>317</v>
-      </c>
-      <c r="E86" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
-        <v>318</v>
-      </c>
-      <c r="B87" t="s">
-        <v>319</v>
-      </c>
-      <c r="C87" t="s">
-        <v>19</v>
-      </c>
-      <c r="D87" t="s">
-        <v>320</v>
-      </c>
-      <c r="E87" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
-        <v>321</v>
-      </c>
-      <c r="B88" t="s">
-        <v>322</v>
-      </c>
-      <c r="C88" t="s">
-        <v>19</v>
-      </c>
-      <c r="D88" t="s">
-        <v>323</v>
-      </c>
-      <c r="E88" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
-        <v>324</v>
-      </c>
-      <c r="B89" t="s">
-        <v>325</v>
-      </c>
-      <c r="C89" t="s">
-        <v>19</v>
-      </c>
-      <c r="D89" t="s">
-        <v>326</v>
-      </c>
-      <c r="E89" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
-        <v>327</v>
-      </c>
-      <c r="B90" t="s">
-        <v>328</v>
-      </c>
-      <c r="C90" t="s">
-        <v>19</v>
-      </c>
-      <c r="D90" t="s">
-        <v>329</v>
-      </c>
-      <c r="E90" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>330</v>
-      </c>
-      <c r="B91" t="s">
-        <v>331</v>
-      </c>
-      <c r="C91" t="s">
-        <v>19</v>
-      </c>
-      <c r="D91" t="s">
-        <v>332</v>
-      </c>
-      <c r="E91" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A92" t="s">
-        <v>333</v>
-      </c>
-      <c r="B92" t="s">
-        <v>334</v>
-      </c>
-      <c r="C92" t="s">
-        <v>35</v>
-      </c>
-      <c r="D92" t="s">
-        <v>335</v>
-      </c>
-      <c r="E92" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
-        <v>336</v>
-      </c>
-      <c r="B93" t="s">
-        <v>337</v>
-      </c>
-      <c r="C93" t="s">
-        <v>19</v>
-      </c>
-      <c r="D93" t="s">
-        <v>338</v>
-      </c>
-      <c r="E93" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
-        <v>339</v>
-      </c>
-      <c r="B94" t="s">
-        <v>340</v>
-      </c>
-      <c r="C94" t="s">
-        <v>46</v>
-      </c>
-      <c r="D94" t="s">
-        <v>341</v>
-      </c>
-      <c r="E94" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
-        <v>342</v>
-      </c>
-      <c r="B95" t="s">
-        <v>343</v>
-      </c>
-      <c r="C95" t="s">
-        <v>46</v>
-      </c>
-      <c r="D95" t="s">
-        <v>344</v>
-      </c>
-      <c r="E95" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
-        <v>114</v>
-      </c>
-      <c r="B96" t="s">
-        <v>115</v>
-      </c>
-      <c r="C96" t="s">
-        <v>19</v>
-      </c>
-      <c r="D96" t="s">
-        <v>345</v>
-      </c>
-      <c r="E96" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
-        <v>346</v>
-      </c>
-      <c r="B97" t="s">
-        <v>347</v>
-      </c>
-      <c r="C97" t="s">
-        <v>46</v>
-      </c>
-      <c r="D97" t="s">
-        <v>348</v>
-      </c>
-      <c r="E97" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
-        <v>349</v>
-      </c>
-      <c r="B98" t="s">
-        <v>350</v>
-      </c>
-      <c r="C98" t="s">
-        <v>46</v>
-      </c>
-      <c r="D98" t="s">
-        <v>351</v>
-      </c>
-      <c r="E98" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
-        <v>352</v>
-      </c>
-      <c r="B99" t="s">
-        <v>353</v>
-      </c>
-      <c r="C99" t="s">
-        <v>46</v>
-      </c>
-      <c r="D99" t="s">
-        <v>354</v>
-      </c>
-      <c r="E99" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
-        <v>352</v>
-      </c>
-      <c r="B100" t="s">
-        <v>353</v>
-      </c>
-      <c r="C100" t="s">
-        <v>46</v>
-      </c>
-      <c r="D100" t="s">
-        <v>355</v>
-      </c>
-      <c r="E100" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
-        <v>352</v>
-      </c>
-      <c r="B101" t="s">
-        <v>353</v>
-      </c>
-      <c r="C101" t="s">
-        <v>46</v>
-      </c>
-      <c r="D101" t="s">
-        <v>356</v>
-      </c>
-      <c r="E101" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A102" t="s">
-        <v>352</v>
-      </c>
-      <c r="B102" t="s">
-        <v>353</v>
-      </c>
-      <c r="C102" t="s">
-        <v>46</v>
-      </c>
-      <c r="D102" t="s">
-        <v>357</v>
-      </c>
-      <c r="E102" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
-        <v>358</v>
-      </c>
-      <c r="B103" t="s">
-        <v>359</v>
-      </c>
-      <c r="C103" t="s">
-        <v>46</v>
-      </c>
-      <c r="D103" t="s">
-        <v>360</v>
-      </c>
-      <c r="E103" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
-        <v>361</v>
-      </c>
-      <c r="B104" t="s">
-        <v>362</v>
-      </c>
-      <c r="C104" t="s">
-        <v>46</v>
-      </c>
-      <c r="D104" t="s">
-        <v>363</v>
-      </c>
-      <c r="E104" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
-        <v>364</v>
-      </c>
-      <c r="B105" t="s">
-        <v>365</v>
-      </c>
-      <c r="C105" t="s">
-        <v>46</v>
-      </c>
-      <c r="D105" t="s">
-        <v>366</v>
-      </c>
-      <c r="E105" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A106" t="s">
-        <v>367</v>
-      </c>
-      <c r="B106" t="s">
-        <v>368</v>
-      </c>
-      <c r="C106" t="s">
-        <v>46</v>
-      </c>
-      <c r="D106" t="s">
-        <v>369</v>
-      </c>
-      <c r="E106" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A107" t="s">
-        <v>370</v>
-      </c>
-      <c r="B107" t="s">
-        <v>371</v>
-      </c>
-      <c r="C107" t="s">
-        <v>46</v>
-      </c>
-      <c r="D107" t="s">
-        <v>372</v>
-      </c>
-      <c r="E107" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A108" t="s">
-        <v>373</v>
-      </c>
-      <c r="B108" t="s">
-        <v>374</v>
-      </c>
-      <c r="C108" t="s">
-        <v>46</v>
-      </c>
-      <c r="D108" t="s">
-        <v>375</v>
-      </c>
-      <c r="E108" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A109" t="s">
-        <v>376</v>
-      </c>
-      <c r="B109" t="s">
-        <v>377</v>
-      </c>
-      <c r="C109" t="s">
-        <v>46</v>
-      </c>
-      <c r="D109" t="s">
-        <v>378</v>
-      </c>
-      <c r="E109" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A110" t="s">
-        <v>380</v>
-      </c>
-      <c r="B110" t="s">
-        <v>381</v>
-      </c>
-      <c r="C110" t="s">
-        <v>46</v>
-      </c>
-      <c r="D110" t="s">
-        <v>382</v>
-      </c>
-      <c r="E110" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A111" t="s">
-        <v>383</v>
-      </c>
-      <c r="B111" t="s">
-        <v>384</v>
-      </c>
-      <c r="C111" t="s">
-        <v>46</v>
-      </c>
-      <c r="D111" t="s">
-        <v>385</v>
-      </c>
-      <c r="E111" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A112" t="s">
-        <v>386</v>
-      </c>
-      <c r="B112" t="s">
-        <v>387</v>
-      </c>
-      <c r="C112" t="s">
-        <v>46</v>
-      </c>
-      <c r="D112" t="s">
-        <v>388</v>
-      </c>
-      <c r="E112" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A113" t="s">
-        <v>389</v>
-      </c>
-      <c r="B113" t="s">
-        <v>390</v>
-      </c>
-      <c r="C113" t="s">
-        <v>46</v>
-      </c>
-      <c r="D113" t="s">
-        <v>391</v>
-      </c>
-      <c r="E113" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A114" t="s">
-        <v>392</v>
-      </c>
-      <c r="B114" t="s">
-        <v>393</v>
-      </c>
-      <c r="C114" t="s">
-        <v>46</v>
-      </c>
-      <c r="D114" t="s">
-        <v>394</v>
-      </c>
-      <c r="E114" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A115" t="s">
-        <v>395</v>
-      </c>
-      <c r="B115" t="s">
-        <v>396</v>
-      </c>
-      <c r="C115" t="s">
-        <v>46</v>
-      </c>
-      <c r="D115" t="s">
-        <v>397</v>
-      </c>
-      <c r="E115" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
-        <v>398</v>
-      </c>
-      <c r="B116" t="s">
-        <v>399</v>
-      </c>
-      <c r="C116" t="s">
-        <v>46</v>
-      </c>
-      <c r="D116" t="s">
-        <v>400</v>
-      </c>
-      <c r="E116" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
-        <v>401</v>
-      </c>
-      <c r="B117" t="s">
-        <v>402</v>
-      </c>
-      <c r="C117" t="s">
-        <v>46</v>
-      </c>
-      <c r="D117" t="s">
-        <v>403</v>
-      </c>
-      <c r="E117" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
-        <v>404</v>
-      </c>
-      <c r="B118" t="s">
-        <v>405</v>
-      </c>
-      <c r="C118" t="s">
-        <v>46</v>
-      </c>
-      <c r="D118" t="s">
-        <v>406</v>
-      </c>
-      <c r="E118" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
-        <v>407</v>
-      </c>
-      <c r="B119" t="s">
-        <v>408</v>
-      </c>
-      <c r="C119" t="s">
-        <v>46</v>
-      </c>
-      <c r="D119" t="s">
-        <v>409</v>
-      </c>
-      <c r="E119" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A120" t="s">
-        <v>410</v>
-      </c>
-      <c r="B120" t="s">
-        <v>411</v>
-      </c>
-      <c r="C120" t="s">
-        <v>46</v>
-      </c>
-      <c r="D120" t="s">
-        <v>412</v>
-      </c>
-      <c r="E120" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A121" t="s">
-        <v>413</v>
-      </c>
-      <c r="B121" t="s">
-        <v>414</v>
-      </c>
-      <c r="C121" t="s">
-        <v>46</v>
-      </c>
-      <c r="D121" t="s">
-        <v>415</v>
-      </c>
-      <c r="E121" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A122" t="s">
-        <v>416</v>
-      </c>
-      <c r="B122" t="s">
-        <v>417</v>
-      </c>
-      <c r="C122" t="s">
-        <v>46</v>
-      </c>
-      <c r="D122" t="s">
-        <v>418</v>
-      </c>
-      <c r="E122" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A123" t="s">
-        <v>419</v>
-      </c>
-      <c r="B123" t="s">
-        <v>420</v>
-      </c>
-      <c r="C123" t="s">
-        <v>46</v>
-      </c>
-      <c r="D123" t="s">
-        <v>421</v>
-      </c>
-      <c r="E123" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A124" t="s">
-        <v>422</v>
-      </c>
-      <c r="B124" t="s">
-        <v>423</v>
-      </c>
-      <c r="C124" t="s">
-        <v>46</v>
-      </c>
-      <c r="D124" t="s">
-        <v>424</v>
-      </c>
-      <c r="E124" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A125" t="s">
-        <v>425</v>
-      </c>
-      <c r="B125" t="s">
-        <v>426</v>
-      </c>
-      <c r="C125" t="s">
-        <v>46</v>
-      </c>
-      <c r="D125" t="s">
-        <v>427</v>
-      </c>
-      <c r="E125" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A126" t="s">
-        <v>428</v>
-      </c>
-      <c r="B126" t="s">
-        <v>429</v>
-      </c>
-      <c r="C126" t="s">
-        <v>46</v>
-      </c>
-      <c r="D126" t="s">
-        <v>430</v>
-      </c>
-      <c r="E126" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A127" t="s">
-        <v>432</v>
-      </c>
-      <c r="B127" t="s">
-        <v>433</v>
-      </c>
-      <c r="C127" t="s">
-        <v>46</v>
-      </c>
-      <c r="D127" t="s">
-        <v>434</v>
-      </c>
-      <c r="E127" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A128" t="s">
-        <v>435</v>
-      </c>
-      <c r="B128" t="s">
-        <v>436</v>
-      </c>
-      <c r="C128" t="s">
-        <v>46</v>
-      </c>
-      <c r="D128" t="s">
-        <v>437</v>
-      </c>
-      <c r="E128" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A129" t="s">
-        <v>438</v>
-      </c>
-      <c r="B129" t="s">
-        <v>439</v>
-      </c>
-      <c r="C129" t="s">
-        <v>46</v>
-      </c>
-      <c r="D129" t="s">
-        <v>440</v>
-      </c>
-      <c r="E129" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A130" t="s">
-        <v>441</v>
-      </c>
-      <c r="B130" t="s">
-        <v>442</v>
-      </c>
-      <c r="C130" t="s">
-        <v>46</v>
-      </c>
-      <c r="D130" t="s">
-        <v>443</v>
-      </c>
-      <c r="E130" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A131" t="s">
-        <v>444</v>
-      </c>
-      <c r="B131" t="s">
-        <v>445</v>
-      </c>
-      <c r="C131" t="s">
-        <v>46</v>
-      </c>
-      <c r="D131" t="s">
-        <v>446</v>
-      </c>
-      <c r="E131" t="s">
-        <v>147</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>